<commit_message>
feat: add IT status (FMIS/eMeeting/Software/Phonebook) support to Excel import
- HEADER_MAP: add fmis/emeeting/software/phonebook column name mappings
- parseITStatusForImport: new helper that returns undefined for blank cells
  (blank = skip existing value) vs explicit status values
- CREATE: auto-fill date to today when status is 'ดำเนินการแล้ว'
- UPDATE: process IT status columns per row — blank skips, explicit value
  updates status + handles date (keep existing date if done, clear if not)
- Import_Template.xlsx: add FMIS/eMeeting/Software/Phonebook columns (N-Q)
  with hint text in row 2; example row 3 left empty for these columns
- ImportPage: update column description and IT status hint text

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Import_Template.xlsx
+++ b/public/Import_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -52,6 +52,18 @@
     <t>อีเมล</t>
   </si>
   <si>
+    <t>FMIS</t>
+  </si>
+  <si>
+    <t>eMeeting</t>
+  </si>
+  <si>
+    <t>Software</t>
+  </si>
+  <si>
+    <t>Phonebook</t>
+  </si>
+  <si>
     <t>1=สบค., 2=ศล.</t>
   </si>
   <si>
@@ -68,6 +80,9 @@
   </si>
   <si>
     <t>example@email.com</t>
+  </si>
+  <si>
+    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ / ไม่พบบัญชี</t>
   </si>
   <si>
     <t>31/3/2599</t>
@@ -538,7 +553,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M200"/>
+  <dimension ref="A1:Q200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -551,9 +566,10 @@
     <col min="11" max="11" width="30" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="26" customWidth="1"/>
+    <col min="14" max="17" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -593,37 +609,61 @@
       <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="D2" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -634,37 +674,41 @@
         <v>2599</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>25</v>
+      <c r="M3" s="3" t="s">
+        <v>32</v>
       </c>
-      <c r="K3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="M3" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+      <c r="P3" s="3"/>
+      <c r="Q3" s="3"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -678,8 +722,12 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="Q4" s="3"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -693,8 +741,12 @@
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
       <c r="M5" s="3"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="Q5" s="3"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -708,8 +760,12 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -723,8 +779,12 @@
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
       <c r="M7" s="3"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="Q7" s="3"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -738,8 +798,12 @@
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
       <c r="M8" s="3"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -753,8 +817,12 @@
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
       <c r="M9" s="3"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="Q9" s="3"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -768,8 +836,12 @@
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
       <c r="M10" s="3"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -783,8 +855,12 @@
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
       <c r="M11" s="3"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -798,8 +874,12 @@
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
       <c r="M12" s="3"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -813,8 +893,12 @@
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
       <c r="M13" s="3"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -828,8 +912,12 @@
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
       <c r="M14" s="3"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -843,8 +931,12 @@
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
       <c r="M15" s="3"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -858,8 +950,12 @@
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
       <c r="M16" s="3"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -873,8 +969,12 @@
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
       <c r="M17" s="3"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -888,8 +988,12 @@
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
       <c r="M18" s="3"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -903,8 +1007,12 @@
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
       <c r="M19" s="3"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -918,8 +1026,12 @@
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
       <c r="M20" s="3"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -933,8 +1045,12 @@
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
       <c r="M21" s="3"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -948,8 +1064,12 @@
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
       <c r="M22" s="3"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -963,8 +1083,12 @@
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
       <c r="M23" s="3"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -978,8 +1102,12 @@
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
       <c r="M24" s="3"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -993,8 +1121,12 @@
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
       <c r="M25" s="3"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1008,8 +1140,12 @@
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
       <c r="M26" s="3"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1023,8 +1159,12 @@
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
       <c r="M27" s="3"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1038,8 +1178,12 @@
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
       <c r="M28" s="3"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1053,8 +1197,12 @@
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
       <c r="M29" s="3"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1068,8 +1216,12 @@
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
       <c r="M30" s="3"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1083,8 +1235,12 @@
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
       <c r="M31" s="3"/>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1098,8 +1254,12 @@
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
       <c r="M32" s="3"/>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1113,8 +1273,12 @@
       <c r="K33" s="3"/>
       <c r="L33" s="3"/>
       <c r="M33" s="3"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+      <c r="P33" s="3"/>
+      <c r="Q33" s="3"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1128,8 +1292,12 @@
       <c r="K34" s="3"/>
       <c r="L34" s="3"/>
       <c r="M34" s="3"/>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+      <c r="P34" s="3"/>
+      <c r="Q34" s="3"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1143,8 +1311,12 @@
       <c r="K35" s="3"/>
       <c r="L35" s="3"/>
       <c r="M35" s="3"/>
-    </row>
-    <row r="36" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+      <c r="P35" s="3"/>
+      <c r="Q35" s="3"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1158,8 +1330,12 @@
       <c r="K36" s="3"/>
       <c r="L36" s="3"/>
       <c r="M36" s="3"/>
-    </row>
-    <row r="37" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+      <c r="P36" s="3"/>
+      <c r="Q36" s="3"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1173,8 +1349,12 @@
       <c r="K37" s="3"/>
       <c r="L37" s="3"/>
       <c r="M37" s="3"/>
-    </row>
-    <row r="38" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+      <c r="P37" s="3"/>
+      <c r="Q37" s="3"/>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1188,8 +1368,12 @@
       <c r="K38" s="3"/>
       <c r="L38" s="3"/>
       <c r="M38" s="3"/>
-    </row>
-    <row r="39" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+      <c r="P38" s="3"/>
+      <c r="Q38" s="3"/>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1203,8 +1387,12 @@
       <c r="K39" s="3"/>
       <c r="L39" s="3"/>
       <c r="M39" s="3"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N39" s="3"/>
+      <c r="O39" s="3"/>
+      <c r="P39" s="3"/>
+      <c r="Q39" s="3"/>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1218,8 +1406,12 @@
       <c r="K40" s="3"/>
       <c r="L40" s="3"/>
       <c r="M40" s="3"/>
-    </row>
-    <row r="41" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N40" s="3"/>
+      <c r="O40" s="3"/>
+      <c r="P40" s="3"/>
+      <c r="Q40" s="3"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1233,8 +1425,12 @@
       <c r="K41" s="3"/>
       <c r="L41" s="3"/>
       <c r="M41" s="3"/>
-    </row>
-    <row r="42" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
+      <c r="P41" s="3"/>
+      <c r="Q41" s="3"/>
+    </row>
+    <row r="42" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1248,8 +1444,12 @@
       <c r="K42" s="3"/>
       <c r="L42" s="3"/>
       <c r="M42" s="3"/>
-    </row>
-    <row r="43" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+      <c r="P42" s="3"/>
+      <c r="Q42" s="3"/>
+    </row>
+    <row r="43" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1263,8 +1463,12 @@
       <c r="K43" s="3"/>
       <c r="L43" s="3"/>
       <c r="M43" s="3"/>
-    </row>
-    <row r="44" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+      <c r="P43" s="3"/>
+      <c r="Q43" s="3"/>
+    </row>
+    <row r="44" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1278,8 +1482,12 @@
       <c r="K44" s="3"/>
       <c r="L44" s="3"/>
       <c r="M44" s="3"/>
-    </row>
-    <row r="45" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+      <c r="P44" s="3"/>
+      <c r="Q44" s="3"/>
+    </row>
+    <row r="45" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1293,8 +1501,12 @@
       <c r="K45" s="3"/>
       <c r="L45" s="3"/>
       <c r="M45" s="3"/>
-    </row>
-    <row r="46" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+      <c r="P45" s="3"/>
+      <c r="Q45" s="3"/>
+    </row>
+    <row r="46" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1308,8 +1520,12 @@
       <c r="K46" s="3"/>
       <c r="L46" s="3"/>
       <c r="M46" s="3"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+      <c r="P46" s="3"/>
+      <c r="Q46" s="3"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1323,8 +1539,12 @@
       <c r="K47" s="3"/>
       <c r="L47" s="3"/>
       <c r="M47" s="3"/>
-    </row>
-    <row r="48" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+      <c r="P47" s="3"/>
+      <c r="Q47" s="3"/>
+    </row>
+    <row r="48" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1338,8 +1558,12 @@
       <c r="K48" s="3"/>
       <c r="L48" s="3"/>
       <c r="M48" s="3"/>
-    </row>
-    <row r="49" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+      <c r="P48" s="3"/>
+      <c r="Q48" s="3"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1353,8 +1577,12 @@
       <c r="K49" s="3"/>
       <c r="L49" s="3"/>
       <c r="M49" s="3"/>
-    </row>
-    <row r="50" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+      <c r="P49" s="3"/>
+      <c r="Q49" s="3"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1368,8 +1596,12 @@
       <c r="K50" s="3"/>
       <c r="L50" s="3"/>
       <c r="M50" s="3"/>
-    </row>
-    <row r="51" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+      <c r="P50" s="3"/>
+      <c r="Q50" s="3"/>
+    </row>
+    <row r="51" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1383,8 +1615,12 @@
       <c r="K51" s="3"/>
       <c r="L51" s="3"/>
       <c r="M51" s="3"/>
-    </row>
-    <row r="52" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+      <c r="P51" s="3"/>
+      <c r="Q51" s="3"/>
+    </row>
+    <row r="52" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1398,8 +1634,12 @@
       <c r="K52" s="3"/>
       <c r="L52" s="3"/>
       <c r="M52" s="3"/>
-    </row>
-    <row r="53" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
+      <c r="P52" s="3"/>
+      <c r="Q52" s="3"/>
+    </row>
+    <row r="53" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1413,8 +1653,12 @@
       <c r="K53" s="3"/>
       <c r="L53" s="3"/>
       <c r="M53" s="3"/>
-    </row>
-    <row r="54" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N53" s="3"/>
+      <c r="O53" s="3"/>
+      <c r="P53" s="3"/>
+      <c r="Q53" s="3"/>
+    </row>
+    <row r="54" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1428,8 +1672,12 @@
       <c r="K54" s="3"/>
       <c r="L54" s="3"/>
       <c r="M54" s="3"/>
-    </row>
-    <row r="55" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N54" s="3"/>
+      <c r="O54" s="3"/>
+      <c r="P54" s="3"/>
+      <c r="Q54" s="3"/>
+    </row>
+    <row r="55" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1443,8 +1691,12 @@
       <c r="K55" s="3"/>
       <c r="L55" s="3"/>
       <c r="M55" s="3"/>
-    </row>
-    <row r="56" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N55" s="3"/>
+      <c r="O55" s="3"/>
+      <c r="P55" s="3"/>
+      <c r="Q55" s="3"/>
+    </row>
+    <row r="56" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1458,8 +1710,12 @@
       <c r="K56" s="3"/>
       <c r="L56" s="3"/>
       <c r="M56" s="3"/>
-    </row>
-    <row r="57" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N56" s="3"/>
+      <c r="O56" s="3"/>
+      <c r="P56" s="3"/>
+      <c r="Q56" s="3"/>
+    </row>
+    <row r="57" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1473,8 +1729,12 @@
       <c r="K57" s="3"/>
       <c r="L57" s="3"/>
       <c r="M57" s="3"/>
-    </row>
-    <row r="58" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N57" s="3"/>
+      <c r="O57" s="3"/>
+      <c r="P57" s="3"/>
+      <c r="Q57" s="3"/>
+    </row>
+    <row r="58" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1488,8 +1748,12 @@
       <c r="K58" s="3"/>
       <c r="L58" s="3"/>
       <c r="M58" s="3"/>
-    </row>
-    <row r="59" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N58" s="3"/>
+      <c r="O58" s="3"/>
+      <c r="P58" s="3"/>
+      <c r="Q58" s="3"/>
+    </row>
+    <row r="59" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1503,8 +1767,12 @@
       <c r="K59" s="3"/>
       <c r="L59" s="3"/>
       <c r="M59" s="3"/>
-    </row>
-    <row r="60" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N59" s="3"/>
+      <c r="O59" s="3"/>
+      <c r="P59" s="3"/>
+      <c r="Q59" s="3"/>
+    </row>
+    <row r="60" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1518,8 +1786,12 @@
       <c r="K60" s="3"/>
       <c r="L60" s="3"/>
       <c r="M60" s="3"/>
-    </row>
-    <row r="61" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N60" s="3"/>
+      <c r="O60" s="3"/>
+      <c r="P60" s="3"/>
+      <c r="Q60" s="3"/>
+    </row>
+    <row r="61" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1533,8 +1805,12 @@
       <c r="K61" s="3"/>
       <c r="L61" s="3"/>
       <c r="M61" s="3"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N61" s="3"/>
+      <c r="O61" s="3"/>
+      <c r="P61" s="3"/>
+      <c r="Q61" s="3"/>
+    </row>
+    <row r="62" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -1548,8 +1824,12 @@
       <c r="K62" s="3"/>
       <c r="L62" s="3"/>
       <c r="M62" s="3"/>
-    </row>
-    <row r="63" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N62" s="3"/>
+      <c r="O62" s="3"/>
+      <c r="P62" s="3"/>
+      <c r="Q62" s="3"/>
+    </row>
+    <row r="63" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1563,8 +1843,12 @@
       <c r="K63" s="3"/>
       <c r="L63" s="3"/>
       <c r="M63" s="3"/>
-    </row>
-    <row r="64" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N63" s="3"/>
+      <c r="O63" s="3"/>
+      <c r="P63" s="3"/>
+      <c r="Q63" s="3"/>
+    </row>
+    <row r="64" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -1578,8 +1862,12 @@
       <c r="K64" s="3"/>
       <c r="L64" s="3"/>
       <c r="M64" s="3"/>
-    </row>
-    <row r="65" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N64" s="3"/>
+      <c r="O64" s="3"/>
+      <c r="P64" s="3"/>
+      <c r="Q64" s="3"/>
+    </row>
+    <row r="65" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1593,8 +1881,12 @@
       <c r="K65" s="3"/>
       <c r="L65" s="3"/>
       <c r="M65" s="3"/>
-    </row>
-    <row r="66" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N65" s="3"/>
+      <c r="O65" s="3"/>
+      <c r="P65" s="3"/>
+      <c r="Q65" s="3"/>
+    </row>
+    <row r="66" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -1608,8 +1900,12 @@
       <c r="K66" s="3"/>
       <c r="L66" s="3"/>
       <c r="M66" s="3"/>
-    </row>
-    <row r="67" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N66" s="3"/>
+      <c r="O66" s="3"/>
+      <c r="P66" s="3"/>
+      <c r="Q66" s="3"/>
+    </row>
+    <row r="67" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1623,8 +1919,12 @@
       <c r="K67" s="3"/>
       <c r="L67" s="3"/>
       <c r="M67" s="3"/>
-    </row>
-    <row r="68" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N67" s="3"/>
+      <c r="O67" s="3"/>
+      <c r="P67" s="3"/>
+      <c r="Q67" s="3"/>
+    </row>
+    <row r="68" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -1638,8 +1938,12 @@
       <c r="K68" s="3"/>
       <c r="L68" s="3"/>
       <c r="M68" s="3"/>
-    </row>
-    <row r="69" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N68" s="3"/>
+      <c r="O68" s="3"/>
+      <c r="P68" s="3"/>
+      <c r="Q68" s="3"/>
+    </row>
+    <row r="69" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1653,8 +1957,12 @@
       <c r="K69" s="3"/>
       <c r="L69" s="3"/>
       <c r="M69" s="3"/>
-    </row>
-    <row r="70" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N69" s="3"/>
+      <c r="O69" s="3"/>
+      <c r="P69" s="3"/>
+      <c r="Q69" s="3"/>
+    </row>
+    <row r="70" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -1668,8 +1976,12 @@
       <c r="K70" s="3"/>
       <c r="L70" s="3"/>
       <c r="M70" s="3"/>
-    </row>
-    <row r="71" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N70" s="3"/>
+      <c r="O70" s="3"/>
+      <c r="P70" s="3"/>
+      <c r="Q70" s="3"/>
+    </row>
+    <row r="71" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1683,8 +1995,12 @@
       <c r="K71" s="3"/>
       <c r="L71" s="3"/>
       <c r="M71" s="3"/>
-    </row>
-    <row r="72" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N71" s="3"/>
+      <c r="O71" s="3"/>
+      <c r="P71" s="3"/>
+      <c r="Q71" s="3"/>
+    </row>
+    <row r="72" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -1698,8 +2014,12 @@
       <c r="K72" s="3"/>
       <c r="L72" s="3"/>
       <c r="M72" s="3"/>
-    </row>
-    <row r="73" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N72" s="3"/>
+      <c r="O72" s="3"/>
+      <c r="P72" s="3"/>
+      <c r="Q72" s="3"/>
+    </row>
+    <row r="73" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -1713,8 +2033,12 @@
       <c r="K73" s="3"/>
       <c r="L73" s="3"/>
       <c r="M73" s="3"/>
-    </row>
-    <row r="74" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N73" s="3"/>
+      <c r="O73" s="3"/>
+      <c r="P73" s="3"/>
+      <c r="Q73" s="3"/>
+    </row>
+    <row r="74" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -1728,8 +2052,12 @@
       <c r="K74" s="3"/>
       <c r="L74" s="3"/>
       <c r="M74" s="3"/>
-    </row>
-    <row r="75" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N74" s="3"/>
+      <c r="O74" s="3"/>
+      <c r="P74" s="3"/>
+      <c r="Q74" s="3"/>
+    </row>
+    <row r="75" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -1743,8 +2071,12 @@
       <c r="K75" s="3"/>
       <c r="L75" s="3"/>
       <c r="M75" s="3"/>
-    </row>
-    <row r="76" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N75" s="3"/>
+      <c r="O75" s="3"/>
+      <c r="P75" s="3"/>
+      <c r="Q75" s="3"/>
+    </row>
+    <row r="76" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -1758,8 +2090,12 @@
       <c r="K76" s="3"/>
       <c r="L76" s="3"/>
       <c r="M76" s="3"/>
-    </row>
-    <row r="77" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N76" s="3"/>
+      <c r="O76" s="3"/>
+      <c r="P76" s="3"/>
+      <c r="Q76" s="3"/>
+    </row>
+    <row r="77" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -1773,8 +2109,12 @@
       <c r="K77" s="3"/>
       <c r="L77" s="3"/>
       <c r="M77" s="3"/>
-    </row>
-    <row r="78" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N77" s="3"/>
+      <c r="O77" s="3"/>
+      <c r="P77" s="3"/>
+      <c r="Q77" s="3"/>
+    </row>
+    <row r="78" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -1788,8 +2128,12 @@
       <c r="K78" s="3"/>
       <c r="L78" s="3"/>
       <c r="M78" s="3"/>
-    </row>
-    <row r="79" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N78" s="3"/>
+      <c r="O78" s="3"/>
+      <c r="P78" s="3"/>
+      <c r="Q78" s="3"/>
+    </row>
+    <row r="79" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -1803,8 +2147,12 @@
       <c r="K79" s="3"/>
       <c r="L79" s="3"/>
       <c r="M79" s="3"/>
-    </row>
-    <row r="80" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N79" s="3"/>
+      <c r="O79" s="3"/>
+      <c r="P79" s="3"/>
+      <c r="Q79" s="3"/>
+    </row>
+    <row r="80" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -1818,8 +2166,12 @@
       <c r="K80" s="3"/>
       <c r="L80" s="3"/>
       <c r="M80" s="3"/>
-    </row>
-    <row r="81" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N80" s="3"/>
+      <c r="O80" s="3"/>
+      <c r="P80" s="3"/>
+      <c r="Q80" s="3"/>
+    </row>
+    <row r="81" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -1833,8 +2185,12 @@
       <c r="K81" s="3"/>
       <c r="L81" s="3"/>
       <c r="M81" s="3"/>
-    </row>
-    <row r="82" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N81" s="3"/>
+      <c r="O81" s="3"/>
+      <c r="P81" s="3"/>
+      <c r="Q81" s="3"/>
+    </row>
+    <row r="82" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -1848,8 +2204,12 @@
       <c r="K82" s="3"/>
       <c r="L82" s="3"/>
       <c r="M82" s="3"/>
-    </row>
-    <row r="83" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N82" s="3"/>
+      <c r="O82" s="3"/>
+      <c r="P82" s="3"/>
+      <c r="Q82" s="3"/>
+    </row>
+    <row r="83" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -1863,8 +2223,12 @@
       <c r="K83" s="3"/>
       <c r="L83" s="3"/>
       <c r="M83" s="3"/>
-    </row>
-    <row r="84" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N83" s="3"/>
+      <c r="O83" s="3"/>
+      <c r="P83" s="3"/>
+      <c r="Q83" s="3"/>
+    </row>
+    <row r="84" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -1878,8 +2242,12 @@
       <c r="K84" s="3"/>
       <c r="L84" s="3"/>
       <c r="M84" s="3"/>
-    </row>
-    <row r="85" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N84" s="3"/>
+      <c r="O84" s="3"/>
+      <c r="P84" s="3"/>
+      <c r="Q84" s="3"/>
+    </row>
+    <row r="85" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -1893,8 +2261,12 @@
       <c r="K85" s="3"/>
       <c r="L85" s="3"/>
       <c r="M85" s="3"/>
-    </row>
-    <row r="86" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N85" s="3"/>
+      <c r="O85" s="3"/>
+      <c r="P85" s="3"/>
+      <c r="Q85" s="3"/>
+    </row>
+    <row r="86" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -1908,8 +2280,12 @@
       <c r="K86" s="3"/>
       <c r="L86" s="3"/>
       <c r="M86" s="3"/>
-    </row>
-    <row r="87" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N86" s="3"/>
+      <c r="O86" s="3"/>
+      <c r="P86" s="3"/>
+      <c r="Q86" s="3"/>
+    </row>
+    <row r="87" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -1923,8 +2299,12 @@
       <c r="K87" s="3"/>
       <c r="L87" s="3"/>
       <c r="M87" s="3"/>
-    </row>
-    <row r="88" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N87" s="3"/>
+      <c r="O87" s="3"/>
+      <c r="P87" s="3"/>
+      <c r="Q87" s="3"/>
+    </row>
+    <row r="88" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -1938,8 +2318,12 @@
       <c r="K88" s="3"/>
       <c r="L88" s="3"/>
       <c r="M88" s="3"/>
-    </row>
-    <row r="89" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N88" s="3"/>
+      <c r="O88" s="3"/>
+      <c r="P88" s="3"/>
+      <c r="Q88" s="3"/>
+    </row>
+    <row r="89" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -1953,8 +2337,12 @@
       <c r="K89" s="3"/>
       <c r="L89" s="3"/>
       <c r="M89" s="3"/>
-    </row>
-    <row r="90" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N89" s="3"/>
+      <c r="O89" s="3"/>
+      <c r="P89" s="3"/>
+      <c r="Q89" s="3"/>
+    </row>
+    <row r="90" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -1968,8 +2356,12 @@
       <c r="K90" s="3"/>
       <c r="L90" s="3"/>
       <c r="M90" s="3"/>
-    </row>
-    <row r="91" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N90" s="3"/>
+      <c r="O90" s="3"/>
+      <c r="P90" s="3"/>
+      <c r="Q90" s="3"/>
+    </row>
+    <row r="91" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -1983,8 +2375,12 @@
       <c r="K91" s="3"/>
       <c r="L91" s="3"/>
       <c r="M91" s="3"/>
-    </row>
-    <row r="92" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N91" s="3"/>
+      <c r="O91" s="3"/>
+      <c r="P91" s="3"/>
+      <c r="Q91" s="3"/>
+    </row>
+    <row r="92" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -1998,8 +2394,12 @@
       <c r="K92" s="3"/>
       <c r="L92" s="3"/>
       <c r="M92" s="3"/>
-    </row>
-    <row r="93" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N92" s="3"/>
+      <c r="O92" s="3"/>
+      <c r="P92" s="3"/>
+      <c r="Q92" s="3"/>
+    </row>
+    <row r="93" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -2013,8 +2413,12 @@
       <c r="K93" s="3"/>
       <c r="L93" s="3"/>
       <c r="M93" s="3"/>
-    </row>
-    <row r="94" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N93" s="3"/>
+      <c r="O93" s="3"/>
+      <c r="P93" s="3"/>
+      <c r="Q93" s="3"/>
+    </row>
+    <row r="94" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -2028,8 +2432,12 @@
       <c r="K94" s="3"/>
       <c r="L94" s="3"/>
       <c r="M94" s="3"/>
-    </row>
-    <row r="95" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N94" s="3"/>
+      <c r="O94" s="3"/>
+      <c r="P94" s="3"/>
+      <c r="Q94" s="3"/>
+    </row>
+    <row r="95" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -2043,8 +2451,12 @@
       <c r="K95" s="3"/>
       <c r="L95" s="3"/>
       <c r="M95" s="3"/>
-    </row>
-    <row r="96" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N95" s="3"/>
+      <c r="O95" s="3"/>
+      <c r="P95" s="3"/>
+      <c r="Q95" s="3"/>
+    </row>
+    <row r="96" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -2058,8 +2470,12 @@
       <c r="K96" s="3"/>
       <c r="L96" s="3"/>
       <c r="M96" s="3"/>
-    </row>
-    <row r="97" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N96" s="3"/>
+      <c r="O96" s="3"/>
+      <c r="P96" s="3"/>
+      <c r="Q96" s="3"/>
+    </row>
+    <row r="97" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -2073,8 +2489,12 @@
       <c r="K97" s="3"/>
       <c r="L97" s="3"/>
       <c r="M97" s="3"/>
-    </row>
-    <row r="98" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N97" s="3"/>
+      <c r="O97" s="3"/>
+      <c r="P97" s="3"/>
+      <c r="Q97" s="3"/>
+    </row>
+    <row r="98" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -2088,8 +2508,12 @@
       <c r="K98" s="3"/>
       <c r="L98" s="3"/>
       <c r="M98" s="3"/>
-    </row>
-    <row r="99" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N98" s="3"/>
+      <c r="O98" s="3"/>
+      <c r="P98" s="3"/>
+      <c r="Q98" s="3"/>
+    </row>
+    <row r="99" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -2103,8 +2527,12 @@
       <c r="K99" s="3"/>
       <c r="L99" s="3"/>
       <c r="M99" s="3"/>
-    </row>
-    <row r="100" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N99" s="3"/>
+      <c r="O99" s="3"/>
+      <c r="P99" s="3"/>
+      <c r="Q99" s="3"/>
+    </row>
+    <row r="100" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -2118,8 +2546,12 @@
       <c r="K100" s="3"/>
       <c r="L100" s="3"/>
       <c r="M100" s="3"/>
-    </row>
-    <row r="101" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N100" s="3"/>
+      <c r="O100" s="3"/>
+      <c r="P100" s="3"/>
+      <c r="Q100" s="3"/>
+    </row>
+    <row r="101" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -2133,8 +2565,12 @@
       <c r="K101" s="3"/>
       <c r="L101" s="3"/>
       <c r="M101" s="3"/>
-    </row>
-    <row r="102" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N101" s="3"/>
+      <c r="O101" s="3"/>
+      <c r="P101" s="3"/>
+      <c r="Q101" s="3"/>
+    </row>
+    <row r="102" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -2148,8 +2584,12 @@
       <c r="K102" s="3"/>
       <c r="L102" s="3"/>
       <c r="M102" s="3"/>
-    </row>
-    <row r="103" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N102" s="3"/>
+      <c r="O102" s="3"/>
+      <c r="P102" s="3"/>
+      <c r="Q102" s="3"/>
+    </row>
+    <row r="103" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -2163,8 +2603,12 @@
       <c r="K103" s="3"/>
       <c r="L103" s="3"/>
       <c r="M103" s="3"/>
-    </row>
-    <row r="104" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N103" s="3"/>
+      <c r="O103" s="3"/>
+      <c r="P103" s="3"/>
+      <c r="Q103" s="3"/>
+    </row>
+    <row r="104" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -2178,8 +2622,12 @@
       <c r="K104" s="3"/>
       <c r="L104" s="3"/>
       <c r="M104" s="3"/>
-    </row>
-    <row r="105" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N104" s="3"/>
+      <c r="O104" s="3"/>
+      <c r="P104" s="3"/>
+      <c r="Q104" s="3"/>
+    </row>
+    <row r="105" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -2193,8 +2641,12 @@
       <c r="K105" s="3"/>
       <c r="L105" s="3"/>
       <c r="M105" s="3"/>
-    </row>
-    <row r="106" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N105" s="3"/>
+      <c r="O105" s="3"/>
+      <c r="P105" s="3"/>
+      <c r="Q105" s="3"/>
+    </row>
+    <row r="106" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -2208,8 +2660,12 @@
       <c r="K106" s="3"/>
       <c r="L106" s="3"/>
       <c r="M106" s="3"/>
-    </row>
-    <row r="107" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N106" s="3"/>
+      <c r="O106" s="3"/>
+      <c r="P106" s="3"/>
+      <c r="Q106" s="3"/>
+    </row>
+    <row r="107" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -2223,8 +2679,12 @@
       <c r="K107" s="3"/>
       <c r="L107" s="3"/>
       <c r="M107" s="3"/>
-    </row>
-    <row r="108" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N107" s="3"/>
+      <c r="O107" s="3"/>
+      <c r="P107" s="3"/>
+      <c r="Q107" s="3"/>
+    </row>
+    <row r="108" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -2238,8 +2698,12 @@
       <c r="K108" s="3"/>
       <c r="L108" s="3"/>
       <c r="M108" s="3"/>
-    </row>
-    <row r="109" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N108" s="3"/>
+      <c r="O108" s="3"/>
+      <c r="P108" s="3"/>
+      <c r="Q108" s="3"/>
+    </row>
+    <row r="109" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -2253,8 +2717,12 @@
       <c r="K109" s="3"/>
       <c r="L109" s="3"/>
       <c r="M109" s="3"/>
-    </row>
-    <row r="110" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N109" s="3"/>
+      <c r="O109" s="3"/>
+      <c r="P109" s="3"/>
+      <c r="Q109" s="3"/>
+    </row>
+    <row r="110" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -2268,8 +2736,12 @@
       <c r="K110" s="3"/>
       <c r="L110" s="3"/>
       <c r="M110" s="3"/>
-    </row>
-    <row r="111" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N110" s="3"/>
+      <c r="O110" s="3"/>
+      <c r="P110" s="3"/>
+      <c r="Q110" s="3"/>
+    </row>
+    <row r="111" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -2283,8 +2755,12 @@
       <c r="K111" s="3"/>
       <c r="L111" s="3"/>
       <c r="M111" s="3"/>
-    </row>
-    <row r="112" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N111" s="3"/>
+      <c r="O111" s="3"/>
+      <c r="P111" s="3"/>
+      <c r="Q111" s="3"/>
+    </row>
+    <row r="112" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -2298,8 +2774,12 @@
       <c r="K112" s="3"/>
       <c r="L112" s="3"/>
       <c r="M112" s="3"/>
-    </row>
-    <row r="113" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N112" s="3"/>
+      <c r="O112" s="3"/>
+      <c r="P112" s="3"/>
+      <c r="Q112" s="3"/>
+    </row>
+    <row r="113" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -2313,8 +2793,12 @@
       <c r="K113" s="3"/>
       <c r="L113" s="3"/>
       <c r="M113" s="3"/>
-    </row>
-    <row r="114" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N113" s="3"/>
+      <c r="O113" s="3"/>
+      <c r="P113" s="3"/>
+      <c r="Q113" s="3"/>
+    </row>
+    <row r="114" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -2328,8 +2812,12 @@
       <c r="K114" s="3"/>
       <c r="L114" s="3"/>
       <c r="M114" s="3"/>
-    </row>
-    <row r="115" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N114" s="3"/>
+      <c r="O114" s="3"/>
+      <c r="P114" s="3"/>
+      <c r="Q114" s="3"/>
+    </row>
+    <row r="115" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -2343,8 +2831,12 @@
       <c r="K115" s="3"/>
       <c r="L115" s="3"/>
       <c r="M115" s="3"/>
-    </row>
-    <row r="116" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N115" s="3"/>
+      <c r="O115" s="3"/>
+      <c r="P115" s="3"/>
+      <c r="Q115" s="3"/>
+    </row>
+    <row r="116" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -2358,8 +2850,12 @@
       <c r="K116" s="3"/>
       <c r="L116" s="3"/>
       <c r="M116" s="3"/>
-    </row>
-    <row r="117" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N116" s="3"/>
+      <c r="O116" s="3"/>
+      <c r="P116" s="3"/>
+      <c r="Q116" s="3"/>
+    </row>
+    <row r="117" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -2373,8 +2869,12 @@
       <c r="K117" s="3"/>
       <c r="L117" s="3"/>
       <c r="M117" s="3"/>
-    </row>
-    <row r="118" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N117" s="3"/>
+      <c r="O117" s="3"/>
+      <c r="P117" s="3"/>
+      <c r="Q117" s="3"/>
+    </row>
+    <row r="118" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -2388,8 +2888,12 @@
       <c r="K118" s="3"/>
       <c r="L118" s="3"/>
       <c r="M118" s="3"/>
-    </row>
-    <row r="119" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N118" s="3"/>
+      <c r="O118" s="3"/>
+      <c r="P118" s="3"/>
+      <c r="Q118" s="3"/>
+    </row>
+    <row r="119" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -2403,8 +2907,12 @@
       <c r="K119" s="3"/>
       <c r="L119" s="3"/>
       <c r="M119" s="3"/>
-    </row>
-    <row r="120" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N119" s="3"/>
+      <c r="O119" s="3"/>
+      <c r="P119" s="3"/>
+      <c r="Q119" s="3"/>
+    </row>
+    <row r="120" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -2418,8 +2926,12 @@
       <c r="K120" s="3"/>
       <c r="L120" s="3"/>
       <c r="M120" s="3"/>
-    </row>
-    <row r="121" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N120" s="3"/>
+      <c r="O120" s="3"/>
+      <c r="P120" s="3"/>
+      <c r="Q120" s="3"/>
+    </row>
+    <row r="121" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -2433,8 +2945,12 @@
       <c r="K121" s="3"/>
       <c r="L121" s="3"/>
       <c r="M121" s="3"/>
-    </row>
-    <row r="122" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N121" s="3"/>
+      <c r="O121" s="3"/>
+      <c r="P121" s="3"/>
+      <c r="Q121" s="3"/>
+    </row>
+    <row r="122" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -2448,8 +2964,12 @@
       <c r="K122" s="3"/>
       <c r="L122" s="3"/>
       <c r="M122" s="3"/>
-    </row>
-    <row r="123" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N122" s="3"/>
+      <c r="O122" s="3"/>
+      <c r="P122" s="3"/>
+      <c r="Q122" s="3"/>
+    </row>
+    <row r="123" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -2463,8 +2983,12 @@
       <c r="K123" s="3"/>
       <c r="L123" s="3"/>
       <c r="M123" s="3"/>
-    </row>
-    <row r="124" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N123" s="3"/>
+      <c r="O123" s="3"/>
+      <c r="P123" s="3"/>
+      <c r="Q123" s="3"/>
+    </row>
+    <row r="124" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -2478,8 +3002,12 @@
       <c r="K124" s="3"/>
       <c r="L124" s="3"/>
       <c r="M124" s="3"/>
-    </row>
-    <row r="125" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N124" s="3"/>
+      <c r="O124" s="3"/>
+      <c r="P124" s="3"/>
+      <c r="Q124" s="3"/>
+    </row>
+    <row r="125" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -2493,8 +3021,12 @@
       <c r="K125" s="3"/>
       <c r="L125" s="3"/>
       <c r="M125" s="3"/>
-    </row>
-    <row r="126" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N125" s="3"/>
+      <c r="O125" s="3"/>
+      <c r="P125" s="3"/>
+      <c r="Q125" s="3"/>
+    </row>
+    <row r="126" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -2508,8 +3040,12 @@
       <c r="K126" s="3"/>
       <c r="L126" s="3"/>
       <c r="M126" s="3"/>
-    </row>
-    <row r="127" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N126" s="3"/>
+      <c r="O126" s="3"/>
+      <c r="P126" s="3"/>
+      <c r="Q126" s="3"/>
+    </row>
+    <row r="127" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -2523,8 +3059,12 @@
       <c r="K127" s="3"/>
       <c r="L127" s="3"/>
       <c r="M127" s="3"/>
-    </row>
-    <row r="128" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N127" s="3"/>
+      <c r="O127" s="3"/>
+      <c r="P127" s="3"/>
+      <c r="Q127" s="3"/>
+    </row>
+    <row r="128" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -2538,8 +3078,12 @@
       <c r="K128" s="3"/>
       <c r="L128" s="3"/>
       <c r="M128" s="3"/>
-    </row>
-    <row r="129" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N128" s="3"/>
+      <c r="O128" s="3"/>
+      <c r="P128" s="3"/>
+      <c r="Q128" s="3"/>
+    </row>
+    <row r="129" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -2553,8 +3097,12 @@
       <c r="K129" s="3"/>
       <c r="L129" s="3"/>
       <c r="M129" s="3"/>
-    </row>
-    <row r="130" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N129" s="3"/>
+      <c r="O129" s="3"/>
+      <c r="P129" s="3"/>
+      <c r="Q129" s="3"/>
+    </row>
+    <row r="130" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -2568,8 +3116,12 @@
       <c r="K130" s="3"/>
       <c r="L130" s="3"/>
       <c r="M130" s="3"/>
-    </row>
-    <row r="131" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N130" s="3"/>
+      <c r="O130" s="3"/>
+      <c r="P130" s="3"/>
+      <c r="Q130" s="3"/>
+    </row>
+    <row r="131" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -2583,8 +3135,12 @@
       <c r="K131" s="3"/>
       <c r="L131" s="3"/>
       <c r="M131" s="3"/>
-    </row>
-    <row r="132" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N131" s="3"/>
+      <c r="O131" s="3"/>
+      <c r="P131" s="3"/>
+      <c r="Q131" s="3"/>
+    </row>
+    <row r="132" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -2598,8 +3154,12 @@
       <c r="K132" s="3"/>
       <c r="L132" s="3"/>
       <c r="M132" s="3"/>
-    </row>
-    <row r="133" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N132" s="3"/>
+      <c r="O132" s="3"/>
+      <c r="P132" s="3"/>
+      <c r="Q132" s="3"/>
+    </row>
+    <row r="133" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -2613,8 +3173,12 @@
       <c r="K133" s="3"/>
       <c r="L133" s="3"/>
       <c r="M133" s="3"/>
-    </row>
-    <row r="134" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N133" s="3"/>
+      <c r="O133" s="3"/>
+      <c r="P133" s="3"/>
+      <c r="Q133" s="3"/>
+    </row>
+    <row r="134" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -2628,8 +3192,12 @@
       <c r="K134" s="3"/>
       <c r="L134" s="3"/>
       <c r="M134" s="3"/>
-    </row>
-    <row r="135" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N134" s="3"/>
+      <c r="O134" s="3"/>
+      <c r="P134" s="3"/>
+      <c r="Q134" s="3"/>
+    </row>
+    <row r="135" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -2643,8 +3211,12 @@
       <c r="K135" s="3"/>
       <c r="L135" s="3"/>
       <c r="M135" s="3"/>
-    </row>
-    <row r="136" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N135" s="3"/>
+      <c r="O135" s="3"/>
+      <c r="P135" s="3"/>
+      <c r="Q135" s="3"/>
+    </row>
+    <row r="136" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -2658,8 +3230,12 @@
       <c r="K136" s="3"/>
       <c r="L136" s="3"/>
       <c r="M136" s="3"/>
-    </row>
-    <row r="137" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N136" s="3"/>
+      <c r="O136" s="3"/>
+      <c r="P136" s="3"/>
+      <c r="Q136" s="3"/>
+    </row>
+    <row r="137" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -2673,8 +3249,12 @@
       <c r="K137" s="3"/>
       <c r="L137" s="3"/>
       <c r="M137" s="3"/>
-    </row>
-    <row r="138" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N137" s="3"/>
+      <c r="O137" s="3"/>
+      <c r="P137" s="3"/>
+      <c r="Q137" s="3"/>
+    </row>
+    <row r="138" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -2688,8 +3268,12 @@
       <c r="K138" s="3"/>
       <c r="L138" s="3"/>
       <c r="M138" s="3"/>
-    </row>
-    <row r="139" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N138" s="3"/>
+      <c r="O138" s="3"/>
+      <c r="P138" s="3"/>
+      <c r="Q138" s="3"/>
+    </row>
+    <row r="139" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -2703,8 +3287,12 @@
       <c r="K139" s="3"/>
       <c r="L139" s="3"/>
       <c r="M139" s="3"/>
-    </row>
-    <row r="140" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N139" s="3"/>
+      <c r="O139" s="3"/>
+      <c r="P139" s="3"/>
+      <c r="Q139" s="3"/>
+    </row>
+    <row r="140" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -2718,8 +3306,12 @@
       <c r="K140" s="3"/>
       <c r="L140" s="3"/>
       <c r="M140" s="3"/>
-    </row>
-    <row r="141" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N140" s="3"/>
+      <c r="O140" s="3"/>
+      <c r="P140" s="3"/>
+      <c r="Q140" s="3"/>
+    </row>
+    <row r="141" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -2733,8 +3325,12 @@
       <c r="K141" s="3"/>
       <c r="L141" s="3"/>
       <c r="M141" s="3"/>
-    </row>
-    <row r="142" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N141" s="3"/>
+      <c r="O141" s="3"/>
+      <c r="P141" s="3"/>
+      <c r="Q141" s="3"/>
+    </row>
+    <row r="142" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -2748,8 +3344,12 @@
       <c r="K142" s="3"/>
       <c r="L142" s="3"/>
       <c r="M142" s="3"/>
-    </row>
-    <row r="143" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N142" s="3"/>
+      <c r="O142" s="3"/>
+      <c r="P142" s="3"/>
+      <c r="Q142" s="3"/>
+    </row>
+    <row r="143" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -2763,8 +3363,12 @@
       <c r="K143" s="3"/>
       <c r="L143" s="3"/>
       <c r="M143" s="3"/>
-    </row>
-    <row r="144" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N143" s="3"/>
+      <c r="O143" s="3"/>
+      <c r="P143" s="3"/>
+      <c r="Q143" s="3"/>
+    </row>
+    <row r="144" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -2778,8 +3382,12 @@
       <c r="K144" s="3"/>
       <c r="L144" s="3"/>
       <c r="M144" s="3"/>
-    </row>
-    <row r="145" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N144" s="3"/>
+      <c r="O144" s="3"/>
+      <c r="P144" s="3"/>
+      <c r="Q144" s="3"/>
+    </row>
+    <row r="145" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -2793,8 +3401,12 @@
       <c r="K145" s="3"/>
       <c r="L145" s="3"/>
       <c r="M145" s="3"/>
-    </row>
-    <row r="146" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N145" s="3"/>
+      <c r="O145" s="3"/>
+      <c r="P145" s="3"/>
+      <c r="Q145" s="3"/>
+    </row>
+    <row r="146" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -2808,8 +3420,12 @@
       <c r="K146" s="3"/>
       <c r="L146" s="3"/>
       <c r="M146" s="3"/>
-    </row>
-    <row r="147" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N146" s="3"/>
+      <c r="O146" s="3"/>
+      <c r="P146" s="3"/>
+      <c r="Q146" s="3"/>
+    </row>
+    <row r="147" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -2823,8 +3439,12 @@
       <c r="K147" s="3"/>
       <c r="L147" s="3"/>
       <c r="M147" s="3"/>
-    </row>
-    <row r="148" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N147" s="3"/>
+      <c r="O147" s="3"/>
+      <c r="P147" s="3"/>
+      <c r="Q147" s="3"/>
+    </row>
+    <row r="148" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -2838,8 +3458,12 @@
       <c r="K148" s="3"/>
       <c r="L148" s="3"/>
       <c r="M148" s="3"/>
-    </row>
-    <row r="149" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N148" s="3"/>
+      <c r="O148" s="3"/>
+      <c r="P148" s="3"/>
+      <c r="Q148" s="3"/>
+    </row>
+    <row r="149" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -2853,8 +3477,12 @@
       <c r="K149" s="3"/>
       <c r="L149" s="3"/>
       <c r="M149" s="3"/>
-    </row>
-    <row r="150" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N149" s="3"/>
+      <c r="O149" s="3"/>
+      <c r="P149" s="3"/>
+      <c r="Q149" s="3"/>
+    </row>
+    <row r="150" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -2868,8 +3496,12 @@
       <c r="K150" s="3"/>
       <c r="L150" s="3"/>
       <c r="M150" s="3"/>
-    </row>
-    <row r="151" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N150" s="3"/>
+      <c r="O150" s="3"/>
+      <c r="P150" s="3"/>
+      <c r="Q150" s="3"/>
+    </row>
+    <row r="151" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -2883,8 +3515,12 @@
       <c r="K151" s="3"/>
       <c r="L151" s="3"/>
       <c r="M151" s="3"/>
-    </row>
-    <row r="152" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N151" s="3"/>
+      <c r="O151" s="3"/>
+      <c r="P151" s="3"/>
+      <c r="Q151" s="3"/>
+    </row>
+    <row r="152" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -2898,8 +3534,12 @@
       <c r="K152" s="3"/>
       <c r="L152" s="3"/>
       <c r="M152" s="3"/>
-    </row>
-    <row r="153" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N152" s="3"/>
+      <c r="O152" s="3"/>
+      <c r="P152" s="3"/>
+      <c r="Q152" s="3"/>
+    </row>
+    <row r="153" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -2913,8 +3553,12 @@
       <c r="K153" s="3"/>
       <c r="L153" s="3"/>
       <c r="M153" s="3"/>
-    </row>
-    <row r="154" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N153" s="3"/>
+      <c r="O153" s="3"/>
+      <c r="P153" s="3"/>
+      <c r="Q153" s="3"/>
+    </row>
+    <row r="154" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -2928,8 +3572,12 @@
       <c r="K154" s="3"/>
       <c r="L154" s="3"/>
       <c r="M154" s="3"/>
-    </row>
-    <row r="155" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N154" s="3"/>
+      <c r="O154" s="3"/>
+      <c r="P154" s="3"/>
+      <c r="Q154" s="3"/>
+    </row>
+    <row r="155" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -2943,8 +3591,12 @@
       <c r="K155" s="3"/>
       <c r="L155" s="3"/>
       <c r="M155" s="3"/>
-    </row>
-    <row r="156" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N155" s="3"/>
+      <c r="O155" s="3"/>
+      <c r="P155" s="3"/>
+      <c r="Q155" s="3"/>
+    </row>
+    <row r="156" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -2958,8 +3610,12 @@
       <c r="K156" s="3"/>
       <c r="L156" s="3"/>
       <c r="M156" s="3"/>
-    </row>
-    <row r="157" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N156" s="3"/>
+      <c r="O156" s="3"/>
+      <c r="P156" s="3"/>
+      <c r="Q156" s="3"/>
+    </row>
+    <row r="157" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -2973,8 +3629,12 @@
       <c r="K157" s="3"/>
       <c r="L157" s="3"/>
       <c r="M157" s="3"/>
-    </row>
-    <row r="158" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N157" s="3"/>
+      <c r="O157" s="3"/>
+      <c r="P157" s="3"/>
+      <c r="Q157" s="3"/>
+    </row>
+    <row r="158" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -2988,8 +3648,12 @@
       <c r="K158" s="3"/>
       <c r="L158" s="3"/>
       <c r="M158" s="3"/>
-    </row>
-    <row r="159" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N158" s="3"/>
+      <c r="O158" s="3"/>
+      <c r="P158" s="3"/>
+      <c r="Q158" s="3"/>
+    </row>
+    <row r="159" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -3003,8 +3667,12 @@
       <c r="K159" s="3"/>
       <c r="L159" s="3"/>
       <c r="M159" s="3"/>
-    </row>
-    <row r="160" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N159" s="3"/>
+      <c r="O159" s="3"/>
+      <c r="P159" s="3"/>
+      <c r="Q159" s="3"/>
+    </row>
+    <row r="160" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -3018,8 +3686,12 @@
       <c r="K160" s="3"/>
       <c r="L160" s="3"/>
       <c r="M160" s="3"/>
-    </row>
-    <row r="161" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N160" s="3"/>
+      <c r="O160" s="3"/>
+      <c r="P160" s="3"/>
+      <c r="Q160" s="3"/>
+    </row>
+    <row r="161" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -3033,8 +3705,12 @@
       <c r="K161" s="3"/>
       <c r="L161" s="3"/>
       <c r="M161" s="3"/>
-    </row>
-    <row r="162" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N161" s="3"/>
+      <c r="O161" s="3"/>
+      <c r="P161" s="3"/>
+      <c r="Q161" s="3"/>
+    </row>
+    <row r="162" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -3048,8 +3724,12 @@
       <c r="K162" s="3"/>
       <c r="L162" s="3"/>
       <c r="M162" s="3"/>
-    </row>
-    <row r="163" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N162" s="3"/>
+      <c r="O162" s="3"/>
+      <c r="P162" s="3"/>
+      <c r="Q162" s="3"/>
+    </row>
+    <row r="163" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -3063,8 +3743,12 @@
       <c r="K163" s="3"/>
       <c r="L163" s="3"/>
       <c r="M163" s="3"/>
-    </row>
-    <row r="164" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N163" s="3"/>
+      <c r="O163" s="3"/>
+      <c r="P163" s="3"/>
+      <c r="Q163" s="3"/>
+    </row>
+    <row r="164" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -3078,8 +3762,12 @@
       <c r="K164" s="3"/>
       <c r="L164" s="3"/>
       <c r="M164" s="3"/>
-    </row>
-    <row r="165" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N164" s="3"/>
+      <c r="O164" s="3"/>
+      <c r="P164" s="3"/>
+      <c r="Q164" s="3"/>
+    </row>
+    <row r="165" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -3093,8 +3781,12 @@
       <c r="K165" s="3"/>
       <c r="L165" s="3"/>
       <c r="M165" s="3"/>
-    </row>
-    <row r="166" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N165" s="3"/>
+      <c r="O165" s="3"/>
+      <c r="P165" s="3"/>
+      <c r="Q165" s="3"/>
+    </row>
+    <row r="166" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -3108,8 +3800,12 @@
       <c r="K166" s="3"/>
       <c r="L166" s="3"/>
       <c r="M166" s="3"/>
-    </row>
-    <row r="167" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N166" s="3"/>
+      <c r="O166" s="3"/>
+      <c r="P166" s="3"/>
+      <c r="Q166" s="3"/>
+    </row>
+    <row r="167" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -3123,8 +3819,12 @@
       <c r="K167" s="3"/>
       <c r="L167" s="3"/>
       <c r="M167" s="3"/>
-    </row>
-    <row r="168" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N167" s="3"/>
+      <c r="O167" s="3"/>
+      <c r="P167" s="3"/>
+      <c r="Q167" s="3"/>
+    </row>
+    <row r="168" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -3138,8 +3838,12 @@
       <c r="K168" s="3"/>
       <c r="L168" s="3"/>
       <c r="M168" s="3"/>
-    </row>
-    <row r="169" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N168" s="3"/>
+      <c r="O168" s="3"/>
+      <c r="P168" s="3"/>
+      <c r="Q168" s="3"/>
+    </row>
+    <row r="169" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -3153,8 +3857,12 @@
       <c r="K169" s="3"/>
       <c r="L169" s="3"/>
       <c r="M169" s="3"/>
-    </row>
-    <row r="170" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N169" s="3"/>
+      <c r="O169" s="3"/>
+      <c r="P169" s="3"/>
+      <c r="Q169" s="3"/>
+    </row>
+    <row r="170" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -3168,8 +3876,12 @@
       <c r="K170" s="3"/>
       <c r="L170" s="3"/>
       <c r="M170" s="3"/>
-    </row>
-    <row r="171" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N170" s="3"/>
+      <c r="O170" s="3"/>
+      <c r="P170" s="3"/>
+      <c r="Q170" s="3"/>
+    </row>
+    <row r="171" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -3183,8 +3895,12 @@
       <c r="K171" s="3"/>
       <c r="L171" s="3"/>
       <c r="M171" s="3"/>
-    </row>
-    <row r="172" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N171" s="3"/>
+      <c r="O171" s="3"/>
+      <c r="P171" s="3"/>
+      <c r="Q171" s="3"/>
+    </row>
+    <row r="172" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -3198,8 +3914,12 @@
       <c r="K172" s="3"/>
       <c r="L172" s="3"/>
       <c r="M172" s="3"/>
-    </row>
-    <row r="173" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N172" s="3"/>
+      <c r="O172" s="3"/>
+      <c r="P172" s="3"/>
+      <c r="Q172" s="3"/>
+    </row>
+    <row r="173" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -3213,8 +3933,12 @@
       <c r="K173" s="3"/>
       <c r="L173" s="3"/>
       <c r="M173" s="3"/>
-    </row>
-    <row r="174" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N173" s="3"/>
+      <c r="O173" s="3"/>
+      <c r="P173" s="3"/>
+      <c r="Q173" s="3"/>
+    </row>
+    <row r="174" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -3228,8 +3952,12 @@
       <c r="K174" s="3"/>
       <c r="L174" s="3"/>
       <c r="M174" s="3"/>
-    </row>
-    <row r="175" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N174" s="3"/>
+      <c r="O174" s="3"/>
+      <c r="P174" s="3"/>
+      <c r="Q174" s="3"/>
+    </row>
+    <row r="175" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -3243,8 +3971,12 @@
       <c r="K175" s="3"/>
       <c r="L175" s="3"/>
       <c r="M175" s="3"/>
-    </row>
-    <row r="176" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N175" s="3"/>
+      <c r="O175" s="3"/>
+      <c r="P175" s="3"/>
+      <c r="Q175" s="3"/>
+    </row>
+    <row r="176" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -3258,8 +3990,12 @@
       <c r="K176" s="3"/>
       <c r="L176" s="3"/>
       <c r="M176" s="3"/>
-    </row>
-    <row r="177" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N176" s="3"/>
+      <c r="O176" s="3"/>
+      <c r="P176" s="3"/>
+      <c r="Q176" s="3"/>
+    </row>
+    <row r="177" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -3273,8 +4009,12 @@
       <c r="K177" s="3"/>
       <c r="L177" s="3"/>
       <c r="M177" s="3"/>
-    </row>
-    <row r="178" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N177" s="3"/>
+      <c r="O177" s="3"/>
+      <c r="P177" s="3"/>
+      <c r="Q177" s="3"/>
+    </row>
+    <row r="178" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -3288,8 +4028,12 @@
       <c r="K178" s="3"/>
       <c r="L178" s="3"/>
       <c r="M178" s="3"/>
-    </row>
-    <row r="179" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N178" s="3"/>
+      <c r="O178" s="3"/>
+      <c r="P178" s="3"/>
+      <c r="Q178" s="3"/>
+    </row>
+    <row r="179" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -3303,8 +4047,12 @@
       <c r="K179" s="3"/>
       <c r="L179" s="3"/>
       <c r="M179" s="3"/>
-    </row>
-    <row r="180" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N179" s="3"/>
+      <c r="O179" s="3"/>
+      <c r="P179" s="3"/>
+      <c r="Q179" s="3"/>
+    </row>
+    <row r="180" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -3318,8 +4066,12 @@
       <c r="K180" s="3"/>
       <c r="L180" s="3"/>
       <c r="M180" s="3"/>
-    </row>
-    <row r="181" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N180" s="3"/>
+      <c r="O180" s="3"/>
+      <c r="P180" s="3"/>
+      <c r="Q180" s="3"/>
+    </row>
+    <row r="181" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -3333,8 +4085,12 @@
       <c r="K181" s="3"/>
       <c r="L181" s="3"/>
       <c r="M181" s="3"/>
-    </row>
-    <row r="182" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N181" s="3"/>
+      <c r="O181" s="3"/>
+      <c r="P181" s="3"/>
+      <c r="Q181" s="3"/>
+    </row>
+    <row r="182" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -3348,8 +4104,12 @@
       <c r="K182" s="3"/>
       <c r="L182" s="3"/>
       <c r="M182" s="3"/>
-    </row>
-    <row r="183" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N182" s="3"/>
+      <c r="O182" s="3"/>
+      <c r="P182" s="3"/>
+      <c r="Q182" s="3"/>
+    </row>
+    <row r="183" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -3363,8 +4123,12 @@
       <c r="K183" s="3"/>
       <c r="L183" s="3"/>
       <c r="M183" s="3"/>
-    </row>
-    <row r="184" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N183" s="3"/>
+      <c r="O183" s="3"/>
+      <c r="P183" s="3"/>
+      <c r="Q183" s="3"/>
+    </row>
+    <row r="184" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -3378,8 +4142,12 @@
       <c r="K184" s="3"/>
       <c r="L184" s="3"/>
       <c r="M184" s="3"/>
-    </row>
-    <row r="185" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N184" s="3"/>
+      <c r="O184" s="3"/>
+      <c r="P184" s="3"/>
+      <c r="Q184" s="3"/>
+    </row>
+    <row r="185" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -3393,8 +4161,12 @@
       <c r="K185" s="3"/>
       <c r="L185" s="3"/>
       <c r="M185" s="3"/>
-    </row>
-    <row r="186" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N185" s="3"/>
+      <c r="O185" s="3"/>
+      <c r="P185" s="3"/>
+      <c r="Q185" s="3"/>
+    </row>
+    <row r="186" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -3408,8 +4180,12 @@
       <c r="K186" s="3"/>
       <c r="L186" s="3"/>
       <c r="M186" s="3"/>
-    </row>
-    <row r="187" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N186" s="3"/>
+      <c r="O186" s="3"/>
+      <c r="P186" s="3"/>
+      <c r="Q186" s="3"/>
+    </row>
+    <row r="187" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -3423,8 +4199,12 @@
       <c r="K187" s="3"/>
       <c r="L187" s="3"/>
       <c r="M187" s="3"/>
-    </row>
-    <row r="188" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N187" s="3"/>
+      <c r="O187" s="3"/>
+      <c r="P187" s="3"/>
+      <c r="Q187" s="3"/>
+    </row>
+    <row r="188" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -3438,8 +4218,12 @@
       <c r="K188" s="3"/>
       <c r="L188" s="3"/>
       <c r="M188" s="3"/>
-    </row>
-    <row r="189" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N188" s="3"/>
+      <c r="O188" s="3"/>
+      <c r="P188" s="3"/>
+      <c r="Q188" s="3"/>
+    </row>
+    <row r="189" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -3453,8 +4237,12 @@
       <c r="K189" s="3"/>
       <c r="L189" s="3"/>
       <c r="M189" s="3"/>
-    </row>
-    <row r="190" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N189" s="3"/>
+      <c r="O189" s="3"/>
+      <c r="P189" s="3"/>
+      <c r="Q189" s="3"/>
+    </row>
+    <row r="190" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -3468,8 +4256,12 @@
       <c r="K190" s="3"/>
       <c r="L190" s="3"/>
       <c r="M190" s="3"/>
-    </row>
-    <row r="191" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N190" s="3"/>
+      <c r="O190" s="3"/>
+      <c r="P190" s="3"/>
+      <c r="Q190" s="3"/>
+    </row>
+    <row r="191" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -3483,8 +4275,12 @@
       <c r="K191" s="3"/>
       <c r="L191" s="3"/>
       <c r="M191" s="3"/>
-    </row>
-    <row r="192" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N191" s="3"/>
+      <c r="O191" s="3"/>
+      <c r="P191" s="3"/>
+      <c r="Q191" s="3"/>
+    </row>
+    <row r="192" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -3498,8 +4294,12 @@
       <c r="K192" s="3"/>
       <c r="L192" s="3"/>
       <c r="M192" s="3"/>
-    </row>
-    <row r="193" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N192" s="3"/>
+      <c r="O192" s="3"/>
+      <c r="P192" s="3"/>
+      <c r="Q192" s="3"/>
+    </row>
+    <row r="193" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -3513,8 +4313,12 @@
       <c r="K193" s="3"/>
       <c r="L193" s="3"/>
       <c r="M193" s="3"/>
-    </row>
-    <row r="194" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N193" s="3"/>
+      <c r="O193" s="3"/>
+      <c r="P193" s="3"/>
+      <c r="Q193" s="3"/>
+    </row>
+    <row r="194" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -3528,8 +4332,12 @@
       <c r="K194" s="3"/>
       <c r="L194" s="3"/>
       <c r="M194" s="3"/>
-    </row>
-    <row r="195" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N194" s="3"/>
+      <c r="O194" s="3"/>
+      <c r="P194" s="3"/>
+      <c r="Q194" s="3"/>
+    </row>
+    <row r="195" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -3543,8 +4351,12 @@
       <c r="K195" s="3"/>
       <c r="L195" s="3"/>
       <c r="M195" s="3"/>
-    </row>
-    <row r="196" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N195" s="3"/>
+      <c r="O195" s="3"/>
+      <c r="P195" s="3"/>
+      <c r="Q195" s="3"/>
+    </row>
+    <row r="196" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -3558,8 +4370,12 @@
       <c r="K196" s="3"/>
       <c r="L196" s="3"/>
       <c r="M196" s="3"/>
-    </row>
-    <row r="197" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N196" s="3"/>
+      <c r="O196" s="3"/>
+      <c r="P196" s="3"/>
+      <c r="Q196" s="3"/>
+    </row>
+    <row r="197" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -3573,8 +4389,12 @@
       <c r="K197" s="3"/>
       <c r="L197" s="3"/>
       <c r="M197" s="3"/>
-    </row>
-    <row r="198" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N197" s="3"/>
+      <c r="O197" s="3"/>
+      <c r="P197" s="3"/>
+      <c r="Q197" s="3"/>
+    </row>
+    <row r="198" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -3588,8 +4408,12 @@
       <c r="K198" s="3"/>
       <c r="L198" s="3"/>
       <c r="M198" s="3"/>
-    </row>
-    <row r="199" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N198" s="3"/>
+      <c r="O198" s="3"/>
+      <c r="P198" s="3"/>
+      <c r="Q198" s="3"/>
+    </row>
+    <row r="199" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -3603,8 +4427,12 @@
       <c r="K199" s="3"/>
       <c r="L199" s="3"/>
       <c r="M199" s="3"/>
-    </row>
-    <row r="200" ht="20" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N199" s="3"/>
+      <c r="O199" s="3"/>
+      <c r="P199" s="3"/>
+      <c r="Q199" s="3"/>
+    </row>
+    <row r="200" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -3618,6 +4446,10 @@
       <c r="K200" s="3"/>
       <c r="L200" s="3"/>
       <c r="M200" s="3"/>
+      <c r="N200" s="3"/>
+      <c r="O200" s="3"/>
+      <c r="P200" s="3"/>
+      <c r="Q200" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: support custom date in IT status import columns
- HEADER_MAP: add วันที่ FMIS/eMeeting/Software/Phonebook mappings
- CREATE: use provided date if present, else auto-fill today
- UPDATE: use provided date → keep existing → auto-fill today (priority order)
- Import_Template.xlsx: rearrange IT columns to paired layout (N-U)
  N=FMIS, O=วันที่ FMIS, P=eMeeting, Q=วันที่ eMeeting,
  R=Software, S=วันที่ Software, T=Phonebook, U=วันที่ Phonebook

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Import_Template.xlsx
+++ b/public/Import_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -55,13 +55,25 @@
     <t>FMIS</t>
   </si>
   <si>
+    <t>วันที่ FMIS</t>
+  </si>
+  <si>
     <t>eMeeting</t>
+  </si>
+  <si>
+    <t>วันที่ eMeeting</t>
   </si>
   <si>
     <t>Software</t>
   </si>
   <si>
+    <t>วันที่ Software</t>
+  </si>
+  <si>
     <t>Phonebook</t>
+  </si>
+  <si>
+    <t>วันที่ Phonebook</t>
   </si>
   <si>
     <t>1=สบค., 2=ศล.</t>
@@ -82,7 +94,10 @@
     <t>example@email.com</t>
   </si>
   <si>
-    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ / ไม่พบบัญชี</t>
+    <t>ดำเนินการแล้ว / ยังไม่ดำเนินการ</t>
+  </si>
+  <si>
+    <t>วว/ดด/ปปปป (พ.ศ.)</t>
   </si>
   <si>
     <t>31/3/2599</t>
@@ -553,7 +568,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q200"/>
+  <dimension ref="A1:U200"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -566,10 +581,17 @@
     <col min="11" max="11" width="30" customWidth="1"/>
     <col min="12" max="12" width="18" customWidth="1"/>
     <col min="13" max="13" width="26" customWidth="1"/>
-    <col min="14" max="17" width="22" customWidth="1"/>
+    <col min="14" max="14" width="22" customWidth="1"/>
+    <col min="15" max="15" width="18" customWidth="1"/>
+    <col min="16" max="16" width="22" customWidth="1"/>
+    <col min="17" max="17" width="18" customWidth="1"/>
+    <col min="18" max="18" width="22" customWidth="1"/>
+    <col min="19" max="19" width="18" customWidth="1"/>
+    <col min="20" max="20" width="22" customWidth="1"/>
+    <col min="21" max="21" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="24" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -621,49 +643,73 @@
       <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="D2" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="O2" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="P2" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="Q2" s="2" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -674,41 +720,45 @@
         <v>2599</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="I3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="J3" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>24</v>
-      </c>
       <c r="M3" s="3" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R3" s="3"/>
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="U3" s="3"/>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
@@ -726,8 +776,12 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="U4" s="3"/>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
@@ -745,8 +799,12 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="U5" s="3"/>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
@@ -764,8 +822,12 @@
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="U6" s="3"/>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
@@ -783,8 +845,12 @@
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="U7" s="3"/>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
@@ -802,8 +868,12 @@
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="U8" s="3"/>
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
@@ -821,8 +891,12 @@
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="U9" s="3"/>
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -840,8 +914,12 @@
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="3"/>
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -859,8 +937,12 @@
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="3"/>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -878,8 +960,12 @@
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+      <c r="U12" s="3"/>
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -897,8 +983,12 @@
       <c r="O13" s="3"/>
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="3"/>
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -916,8 +1006,12 @@
       <c r="O14" s="3"/>
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="3"/>
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -935,8 +1029,12 @@
       <c r="O15" s="3"/>
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="3"/>
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -954,8 +1052,12 @@
       <c r="O16" s="3"/>
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="3"/>
+    </row>
+    <row r="17" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -973,8 +1075,12 @@
       <c r="O17" s="3"/>
       <c r="P17" s="3"/>
       <c r="Q17" s="3"/>
-    </row>
-    <row r="18" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="3"/>
+    </row>
+    <row r="18" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -992,8 +1098,12 @@
       <c r="O18" s="3"/>
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
-    </row>
-    <row r="19" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="3"/>
+    </row>
+    <row r="19" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -1011,8 +1121,12 @@
       <c r="O19" s="3"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="3"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -1030,8 +1144,12 @@
       <c r="O20" s="3"/>
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="3"/>
+    </row>
+    <row r="21" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -1049,8 +1167,12 @@
       <c r="O21" s="3"/>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="3"/>
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -1068,8 +1190,12 @@
       <c r="O22" s="3"/>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="U22" s="3"/>
+    </row>
+    <row r="23" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -1087,8 +1213,12 @@
       <c r="O23" s="3"/>
       <c r="P23" s="3"/>
       <c r="Q23" s="3"/>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="3"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -1106,8 +1236,12 @@
       <c r="O24" s="3"/>
       <c r="P24" s="3"/>
       <c r="Q24" s="3"/>
-    </row>
-    <row r="25" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+    </row>
+    <row r="25" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -1125,8 +1259,12 @@
       <c r="O25" s="3"/>
       <c r="P25" s="3"/>
       <c r="Q25" s="3"/>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+    </row>
+    <row r="26" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
       <c r="C26" s="3"/>
@@ -1144,8 +1282,12 @@
       <c r="O26" s="3"/>
       <c r="P26" s="3"/>
       <c r="Q26" s="3"/>
-    </row>
-    <row r="27" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="3"/>
+    </row>
+    <row r="27" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -1163,8 +1305,12 @@
       <c r="O27" s="3"/>
       <c r="P27" s="3"/>
       <c r="Q27" s="3"/>
-    </row>
-    <row r="28" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="3"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
       <c r="C28" s="3"/>
@@ -1182,8 +1328,12 @@
       <c r="O28" s="3"/>
       <c r="P28" s="3"/>
       <c r="Q28" s="3"/>
-    </row>
-    <row r="29" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="3"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
       <c r="C29" s="3"/>
@@ -1201,8 +1351,12 @@
       <c r="O29" s="3"/>
       <c r="P29" s="3"/>
       <c r="Q29" s="3"/>
-    </row>
-    <row r="30" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="3"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
       <c r="C30" s="3"/>
@@ -1220,8 +1374,12 @@
       <c r="O30" s="3"/>
       <c r="P30" s="3"/>
       <c r="Q30" s="3"/>
-    </row>
-    <row r="31" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -1239,8 +1397,12 @@
       <c r="O31" s="3"/>
       <c r="P31" s="3"/>
       <c r="Q31" s="3"/>
-    </row>
-    <row r="32" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
+      <c r="U31" s="3"/>
+    </row>
+    <row r="32" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
       <c r="C32" s="3"/>
@@ -1258,8 +1420,12 @@
       <c r="O32" s="3"/>
       <c r="P32" s="3"/>
       <c r="Q32" s="3"/>
-    </row>
-    <row r="33" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="3"/>
+    </row>
+    <row r="33" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
       <c r="C33" s="3"/>
@@ -1277,8 +1443,12 @@
       <c r="O33" s="3"/>
       <c r="P33" s="3"/>
       <c r="Q33" s="3"/>
-    </row>
-    <row r="34" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R33" s="3"/>
+      <c r="S33" s="3"/>
+      <c r="T33" s="3"/>
+      <c r="U33" s="3"/>
+    </row>
+    <row r="34" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
       <c r="C34" s="3"/>
@@ -1296,8 +1466,12 @@
       <c r="O34" s="3"/>
       <c r="P34" s="3"/>
       <c r="Q34" s="3"/>
-    </row>
-    <row r="35" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R34" s="3"/>
+      <c r="S34" s="3"/>
+      <c r="T34" s="3"/>
+      <c r="U34" s="3"/>
+    </row>
+    <row r="35" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
       <c r="C35" s="3"/>
@@ -1315,8 +1489,12 @@
       <c r="O35" s="3"/>
       <c r="P35" s="3"/>
       <c r="Q35" s="3"/>
-    </row>
-    <row r="36" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R35" s="3"/>
+      <c r="S35" s="3"/>
+      <c r="T35" s="3"/>
+      <c r="U35" s="3"/>
+    </row>
+    <row r="36" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
       <c r="C36" s="3"/>
@@ -1334,8 +1512,12 @@
       <c r="O36" s="3"/>
       <c r="P36" s="3"/>
       <c r="Q36" s="3"/>
-    </row>
-    <row r="37" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R36" s="3"/>
+      <c r="S36" s="3"/>
+      <c r="T36" s="3"/>
+      <c r="U36" s="3"/>
+    </row>
+    <row r="37" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="3"/>
       <c r="B37" s="3"/>
       <c r="C37" s="3"/>
@@ -1353,8 +1535,12 @@
       <c r="O37" s="3"/>
       <c r="P37" s="3"/>
       <c r="Q37" s="3"/>
-    </row>
-    <row r="38" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R37" s="3"/>
+      <c r="S37" s="3"/>
+      <c r="T37" s="3"/>
+      <c r="U37" s="3"/>
+    </row>
+    <row r="38" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="3"/>
       <c r="B38" s="3"/>
       <c r="C38" s="3"/>
@@ -1372,8 +1558,12 @@
       <c r="O38" s="3"/>
       <c r="P38" s="3"/>
       <c r="Q38" s="3"/>
-    </row>
-    <row r="39" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R38" s="3"/>
+      <c r="S38" s="3"/>
+      <c r="T38" s="3"/>
+      <c r="U38" s="3"/>
+    </row>
+    <row r="39" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="3"/>
       <c r="B39" s="3"/>
       <c r="C39" s="3"/>
@@ -1391,8 +1581,12 @@
       <c r="O39" s="3"/>
       <c r="P39" s="3"/>
       <c r="Q39" s="3"/>
-    </row>
-    <row r="40" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R39" s="3"/>
+      <c r="S39" s="3"/>
+      <c r="T39" s="3"/>
+      <c r="U39" s="3"/>
+    </row>
+    <row r="40" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="3"/>
       <c r="B40" s="3"/>
       <c r="C40" s="3"/>
@@ -1410,8 +1604,12 @@
       <c r="O40" s="3"/>
       <c r="P40" s="3"/>
       <c r="Q40" s="3"/>
-    </row>
-    <row r="41" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R40" s="3"/>
+      <c r="S40" s="3"/>
+      <c r="T40" s="3"/>
+      <c r="U40" s="3"/>
+    </row>
+    <row r="41" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="3"/>
       <c r="B41" s="3"/>
       <c r="C41" s="3"/>
@@ -1429,8 +1627,12 @@
       <c r="O41" s="3"/>
       <c r="P41" s="3"/>
       <c r="Q41" s="3"/>
-    </row>
-    <row r="42" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R41" s="3"/>
+      <c r="S41" s="3"/>
+      <c r="T41" s="3"/>
+      <c r="U41" s="3"/>
+    </row>
+    <row r="42" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="3"/>
       <c r="B42" s="3"/>
       <c r="C42" s="3"/>
@@ -1448,8 +1650,12 @@
       <c r="O42" s="3"/>
       <c r="P42" s="3"/>
       <c r="Q42" s="3"/>
-    </row>
-    <row r="43" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R42" s="3"/>
+      <c r="S42" s="3"/>
+      <c r="T42" s="3"/>
+      <c r="U42" s="3"/>
+    </row>
+    <row r="43" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="3"/>
       <c r="B43" s="3"/>
       <c r="C43" s="3"/>
@@ -1467,8 +1673,12 @@
       <c r="O43" s="3"/>
       <c r="P43" s="3"/>
       <c r="Q43" s="3"/>
-    </row>
-    <row r="44" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R43" s="3"/>
+      <c r="S43" s="3"/>
+      <c r="T43" s="3"/>
+      <c r="U43" s="3"/>
+    </row>
+    <row r="44" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="3"/>
       <c r="B44" s="3"/>
       <c r="C44" s="3"/>
@@ -1486,8 +1696,12 @@
       <c r="O44" s="3"/>
       <c r="P44" s="3"/>
       <c r="Q44" s="3"/>
-    </row>
-    <row r="45" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R44" s="3"/>
+      <c r="S44" s="3"/>
+      <c r="T44" s="3"/>
+      <c r="U44" s="3"/>
+    </row>
+    <row r="45" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="3"/>
       <c r="B45" s="3"/>
       <c r="C45" s="3"/>
@@ -1505,8 +1719,12 @@
       <c r="O45" s="3"/>
       <c r="P45" s="3"/>
       <c r="Q45" s="3"/>
-    </row>
-    <row r="46" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R45" s="3"/>
+      <c r="S45" s="3"/>
+      <c r="T45" s="3"/>
+      <c r="U45" s="3"/>
+    </row>
+    <row r="46" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="3"/>
       <c r="B46" s="3"/>
       <c r="C46" s="3"/>
@@ -1524,8 +1742,12 @@
       <c r="O46" s="3"/>
       <c r="P46" s="3"/>
       <c r="Q46" s="3"/>
-    </row>
-    <row r="47" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R46" s="3"/>
+      <c r="S46" s="3"/>
+      <c r="T46" s="3"/>
+      <c r="U46" s="3"/>
+    </row>
+    <row r="47" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="3"/>
       <c r="B47" s="3"/>
       <c r="C47" s="3"/>
@@ -1543,8 +1765,12 @@
       <c r="O47" s="3"/>
       <c r="P47" s="3"/>
       <c r="Q47" s="3"/>
-    </row>
-    <row r="48" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R47" s="3"/>
+      <c r="S47" s="3"/>
+      <c r="T47" s="3"/>
+      <c r="U47" s="3"/>
+    </row>
+    <row r="48" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="3"/>
       <c r="B48" s="3"/>
       <c r="C48" s="3"/>
@@ -1562,8 +1788,12 @@
       <c r="O48" s="3"/>
       <c r="P48" s="3"/>
       <c r="Q48" s="3"/>
-    </row>
-    <row r="49" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R48" s="3"/>
+      <c r="S48" s="3"/>
+      <c r="T48" s="3"/>
+      <c r="U48" s="3"/>
+    </row>
+    <row r="49" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="3"/>
       <c r="B49" s="3"/>
       <c r="C49" s="3"/>
@@ -1581,8 +1811,12 @@
       <c r="O49" s="3"/>
       <c r="P49" s="3"/>
       <c r="Q49" s="3"/>
-    </row>
-    <row r="50" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R49" s="3"/>
+      <c r="S49" s="3"/>
+      <c r="T49" s="3"/>
+      <c r="U49" s="3"/>
+    </row>
+    <row r="50" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="3"/>
       <c r="B50" s="3"/>
       <c r="C50" s="3"/>
@@ -1600,8 +1834,12 @@
       <c r="O50" s="3"/>
       <c r="P50" s="3"/>
       <c r="Q50" s="3"/>
-    </row>
-    <row r="51" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R50" s="3"/>
+      <c r="S50" s="3"/>
+      <c r="T50" s="3"/>
+      <c r="U50" s="3"/>
+    </row>
+    <row r="51" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="3"/>
       <c r="B51" s="3"/>
       <c r="C51" s="3"/>
@@ -1619,8 +1857,12 @@
       <c r="O51" s="3"/>
       <c r="P51" s="3"/>
       <c r="Q51" s="3"/>
-    </row>
-    <row r="52" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R51" s="3"/>
+      <c r="S51" s="3"/>
+      <c r="T51" s="3"/>
+      <c r="U51" s="3"/>
+    </row>
+    <row r="52" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="3"/>
       <c r="B52" s="3"/>
       <c r="C52" s="3"/>
@@ -1638,8 +1880,12 @@
       <c r="O52" s="3"/>
       <c r="P52" s="3"/>
       <c r="Q52" s="3"/>
-    </row>
-    <row r="53" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R52" s="3"/>
+      <c r="S52" s="3"/>
+      <c r="T52" s="3"/>
+      <c r="U52" s="3"/>
+    </row>
+    <row r="53" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
       <c r="B53" s="3"/>
       <c r="C53" s="3"/>
@@ -1657,8 +1903,12 @@
       <c r="O53" s="3"/>
       <c r="P53" s="3"/>
       <c r="Q53" s="3"/>
-    </row>
-    <row r="54" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R53" s="3"/>
+      <c r="S53" s="3"/>
+      <c r="T53" s="3"/>
+      <c r="U53" s="3"/>
+    </row>
+    <row r="54" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
       <c r="B54" s="3"/>
       <c r="C54" s="3"/>
@@ -1676,8 +1926,12 @@
       <c r="O54" s="3"/>
       <c r="P54" s="3"/>
       <c r="Q54" s="3"/>
-    </row>
-    <row r="55" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R54" s="3"/>
+      <c r="S54" s="3"/>
+      <c r="T54" s="3"/>
+      <c r="U54" s="3"/>
+    </row>
+    <row r="55" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
       <c r="B55" s="3"/>
       <c r="C55" s="3"/>
@@ -1695,8 +1949,12 @@
       <c r="O55" s="3"/>
       <c r="P55" s="3"/>
       <c r="Q55" s="3"/>
-    </row>
-    <row r="56" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R55" s="3"/>
+      <c r="S55" s="3"/>
+      <c r="T55" s="3"/>
+      <c r="U55" s="3"/>
+    </row>
+    <row r="56" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
       <c r="B56" s="3"/>
       <c r="C56" s="3"/>
@@ -1714,8 +1972,12 @@
       <c r="O56" s="3"/>
       <c r="P56" s="3"/>
       <c r="Q56" s="3"/>
-    </row>
-    <row r="57" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R56" s="3"/>
+      <c r="S56" s="3"/>
+      <c r="T56" s="3"/>
+      <c r="U56" s="3"/>
+    </row>
+    <row r="57" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
       <c r="B57" s="3"/>
       <c r="C57" s="3"/>
@@ -1733,8 +1995,12 @@
       <c r="O57" s="3"/>
       <c r="P57" s="3"/>
       <c r="Q57" s="3"/>
-    </row>
-    <row r="58" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R57" s="3"/>
+      <c r="S57" s="3"/>
+      <c r="T57" s="3"/>
+      <c r="U57" s="3"/>
+    </row>
+    <row r="58" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
       <c r="B58" s="3"/>
       <c r="C58" s="3"/>
@@ -1752,8 +2018,12 @@
       <c r="O58" s="3"/>
       <c r="P58" s="3"/>
       <c r="Q58" s="3"/>
-    </row>
-    <row r="59" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R58" s="3"/>
+      <c r="S58" s="3"/>
+      <c r="T58" s="3"/>
+      <c r="U58" s="3"/>
+    </row>
+    <row r="59" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
       <c r="B59" s="3"/>
       <c r="C59" s="3"/>
@@ -1771,8 +2041,12 @@
       <c r="O59" s="3"/>
       <c r="P59" s="3"/>
       <c r="Q59" s="3"/>
-    </row>
-    <row r="60" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R59" s="3"/>
+      <c r="S59" s="3"/>
+      <c r="T59" s="3"/>
+      <c r="U59" s="3"/>
+    </row>
+    <row r="60" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
       <c r="B60" s="3"/>
       <c r="C60" s="3"/>
@@ -1790,8 +2064,12 @@
       <c r="O60" s="3"/>
       <c r="P60" s="3"/>
       <c r="Q60" s="3"/>
-    </row>
-    <row r="61" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R60" s="3"/>
+      <c r="S60" s="3"/>
+      <c r="T60" s="3"/>
+      <c r="U60" s="3"/>
+    </row>
+    <row r="61" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
       <c r="B61" s="3"/>
       <c r="C61" s="3"/>
@@ -1809,8 +2087,12 @@
       <c r="O61" s="3"/>
       <c r="P61" s="3"/>
       <c r="Q61" s="3"/>
-    </row>
-    <row r="62" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R61" s="3"/>
+      <c r="S61" s="3"/>
+      <c r="T61" s="3"/>
+      <c r="U61" s="3"/>
+    </row>
+    <row r="62" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
       <c r="B62" s="3"/>
       <c r="C62" s="3"/>
@@ -1828,8 +2110,12 @@
       <c r="O62" s="3"/>
       <c r="P62" s="3"/>
       <c r="Q62" s="3"/>
-    </row>
-    <row r="63" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R62" s="3"/>
+      <c r="S62" s="3"/>
+      <c r="T62" s="3"/>
+      <c r="U62" s="3"/>
+    </row>
+    <row r="63" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
       <c r="B63" s="3"/>
       <c r="C63" s="3"/>
@@ -1847,8 +2133,12 @@
       <c r="O63" s="3"/>
       <c r="P63" s="3"/>
       <c r="Q63" s="3"/>
-    </row>
-    <row r="64" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R63" s="3"/>
+      <c r="S63" s="3"/>
+      <c r="T63" s="3"/>
+      <c r="U63" s="3"/>
+    </row>
+    <row r="64" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
       <c r="B64" s="3"/>
       <c r="C64" s="3"/>
@@ -1866,8 +2156,12 @@
       <c r="O64" s="3"/>
       <c r="P64" s="3"/>
       <c r="Q64" s="3"/>
-    </row>
-    <row r="65" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R64" s="3"/>
+      <c r="S64" s="3"/>
+      <c r="T64" s="3"/>
+      <c r="U64" s="3"/>
+    </row>
+    <row r="65" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
       <c r="B65" s="3"/>
       <c r="C65" s="3"/>
@@ -1885,8 +2179,12 @@
       <c r="O65" s="3"/>
       <c r="P65" s="3"/>
       <c r="Q65" s="3"/>
-    </row>
-    <row r="66" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R65" s="3"/>
+      <c r="S65" s="3"/>
+      <c r="T65" s="3"/>
+      <c r="U65" s="3"/>
+    </row>
+    <row r="66" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A66" s="3"/>
       <c r="B66" s="3"/>
       <c r="C66" s="3"/>
@@ -1904,8 +2202,12 @@
       <c r="O66" s="3"/>
       <c r="P66" s="3"/>
       <c r="Q66" s="3"/>
-    </row>
-    <row r="67" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R66" s="3"/>
+      <c r="S66" s="3"/>
+      <c r="T66" s="3"/>
+      <c r="U66" s="3"/>
+    </row>
+    <row r="67" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
       <c r="B67" s="3"/>
       <c r="C67" s="3"/>
@@ -1923,8 +2225,12 @@
       <c r="O67" s="3"/>
       <c r="P67" s="3"/>
       <c r="Q67" s="3"/>
-    </row>
-    <row r="68" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R67" s="3"/>
+      <c r="S67" s="3"/>
+      <c r="T67" s="3"/>
+      <c r="U67" s="3"/>
+    </row>
+    <row r="68" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
       <c r="B68" s="3"/>
       <c r="C68" s="3"/>
@@ -1942,8 +2248,12 @@
       <c r="O68" s="3"/>
       <c r="P68" s="3"/>
       <c r="Q68" s="3"/>
-    </row>
-    <row r="69" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R68" s="3"/>
+      <c r="S68" s="3"/>
+      <c r="T68" s="3"/>
+      <c r="U68" s="3"/>
+    </row>
+    <row r="69" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
       <c r="B69" s="3"/>
       <c r="C69" s="3"/>
@@ -1961,8 +2271,12 @@
       <c r="O69" s="3"/>
       <c r="P69" s="3"/>
       <c r="Q69" s="3"/>
-    </row>
-    <row r="70" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R69" s="3"/>
+      <c r="S69" s="3"/>
+      <c r="T69" s="3"/>
+      <c r="U69" s="3"/>
+    </row>
+    <row r="70" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
       <c r="B70" s="3"/>
       <c r="C70" s="3"/>
@@ -1980,8 +2294,12 @@
       <c r="O70" s="3"/>
       <c r="P70" s="3"/>
       <c r="Q70" s="3"/>
-    </row>
-    <row r="71" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R70" s="3"/>
+      <c r="S70" s="3"/>
+      <c r="T70" s="3"/>
+      <c r="U70" s="3"/>
+    </row>
+    <row r="71" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
       <c r="B71" s="3"/>
       <c r="C71" s="3"/>
@@ -1999,8 +2317,12 @@
       <c r="O71" s="3"/>
       <c r="P71" s="3"/>
       <c r="Q71" s="3"/>
-    </row>
-    <row r="72" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R71" s="3"/>
+      <c r="S71" s="3"/>
+      <c r="T71" s="3"/>
+      <c r="U71" s="3"/>
+    </row>
+    <row r="72" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
       <c r="B72" s="3"/>
       <c r="C72" s="3"/>
@@ -2018,8 +2340,12 @@
       <c r="O72" s="3"/>
       <c r="P72" s="3"/>
       <c r="Q72" s="3"/>
-    </row>
-    <row r="73" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R72" s="3"/>
+      <c r="S72" s="3"/>
+      <c r="T72" s="3"/>
+      <c r="U72" s="3"/>
+    </row>
+    <row r="73" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="3"/>
       <c r="C73" s="3"/>
@@ -2037,8 +2363,12 @@
       <c r="O73" s="3"/>
       <c r="P73" s="3"/>
       <c r="Q73" s="3"/>
-    </row>
-    <row r="74" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R73" s="3"/>
+      <c r="S73" s="3"/>
+      <c r="T73" s="3"/>
+      <c r="U73" s="3"/>
+    </row>
+    <row r="74" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="3"/>
       <c r="C74" s="3"/>
@@ -2056,8 +2386,12 @@
       <c r="O74" s="3"/>
       <c r="P74" s="3"/>
       <c r="Q74" s="3"/>
-    </row>
-    <row r="75" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R74" s="3"/>
+      <c r="S74" s="3"/>
+      <c r="T74" s="3"/>
+      <c r="U74" s="3"/>
+    </row>
+    <row r="75" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
       <c r="B75" s="3"/>
       <c r="C75" s="3"/>
@@ -2075,8 +2409,12 @@
       <c r="O75" s="3"/>
       <c r="P75" s="3"/>
       <c r="Q75" s="3"/>
-    </row>
-    <row r="76" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R75" s="3"/>
+      <c r="S75" s="3"/>
+      <c r="T75" s="3"/>
+      <c r="U75" s="3"/>
+    </row>
+    <row r="76" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="3"/>
       <c r="B76" s="3"/>
       <c r="C76" s="3"/>
@@ -2094,8 +2432,12 @@
       <c r="O76" s="3"/>
       <c r="P76" s="3"/>
       <c r="Q76" s="3"/>
-    </row>
-    <row r="77" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R76" s="3"/>
+      <c r="S76" s="3"/>
+      <c r="T76" s="3"/>
+      <c r="U76" s="3"/>
+    </row>
+    <row r="77" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
       <c r="B77" s="3"/>
       <c r="C77" s="3"/>
@@ -2113,8 +2455,12 @@
       <c r="O77" s="3"/>
       <c r="P77" s="3"/>
       <c r="Q77" s="3"/>
-    </row>
-    <row r="78" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R77" s="3"/>
+      <c r="S77" s="3"/>
+      <c r="T77" s="3"/>
+      <c r="U77" s="3"/>
+    </row>
+    <row r="78" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
       <c r="B78" s="3"/>
       <c r="C78" s="3"/>
@@ -2132,8 +2478,12 @@
       <c r="O78" s="3"/>
       <c r="P78" s="3"/>
       <c r="Q78" s="3"/>
-    </row>
-    <row r="79" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R78" s="3"/>
+      <c r="S78" s="3"/>
+      <c r="T78" s="3"/>
+      <c r="U78" s="3"/>
+    </row>
+    <row r="79" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
       <c r="B79" s="3"/>
       <c r="C79" s="3"/>
@@ -2151,8 +2501,12 @@
       <c r="O79" s="3"/>
       <c r="P79" s="3"/>
       <c r="Q79" s="3"/>
-    </row>
-    <row r="80" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R79" s="3"/>
+      <c r="S79" s="3"/>
+      <c r="T79" s="3"/>
+      <c r="U79" s="3"/>
+    </row>
+    <row r="80" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
       <c r="B80" s="3"/>
       <c r="C80" s="3"/>
@@ -2170,8 +2524,12 @@
       <c r="O80" s="3"/>
       <c r="P80" s="3"/>
       <c r="Q80" s="3"/>
-    </row>
-    <row r="81" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R80" s="3"/>
+      <c r="S80" s="3"/>
+      <c r="T80" s="3"/>
+      <c r="U80" s="3"/>
+    </row>
+    <row r="81" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
       <c r="B81" s="3"/>
       <c r="C81" s="3"/>
@@ -2189,8 +2547,12 @@
       <c r="O81" s="3"/>
       <c r="P81" s="3"/>
       <c r="Q81" s="3"/>
-    </row>
-    <row r="82" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R81" s="3"/>
+      <c r="S81" s="3"/>
+      <c r="T81" s="3"/>
+      <c r="U81" s="3"/>
+    </row>
+    <row r="82" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="3"/>
       <c r="C82" s="3"/>
@@ -2208,8 +2570,12 @@
       <c r="O82" s="3"/>
       <c r="P82" s="3"/>
       <c r="Q82" s="3"/>
-    </row>
-    <row r="83" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R82" s="3"/>
+      <c r="S82" s="3"/>
+      <c r="T82" s="3"/>
+      <c r="U82" s="3"/>
+    </row>
+    <row r="83" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="3"/>
       <c r="C83" s="3"/>
@@ -2227,8 +2593,12 @@
       <c r="O83" s="3"/>
       <c r="P83" s="3"/>
       <c r="Q83" s="3"/>
-    </row>
-    <row r="84" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R83" s="3"/>
+      <c r="S83" s="3"/>
+      <c r="T83" s="3"/>
+      <c r="U83" s="3"/>
+    </row>
+    <row r="84" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="3"/>
       <c r="C84" s="3"/>
@@ -2246,8 +2616,12 @@
       <c r="O84" s="3"/>
       <c r="P84" s="3"/>
       <c r="Q84" s="3"/>
-    </row>
-    <row r="85" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R84" s="3"/>
+      <c r="S84" s="3"/>
+      <c r="T84" s="3"/>
+      <c r="U84" s="3"/>
+    </row>
+    <row r="85" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A85" s="3"/>
       <c r="B85" s="3"/>
       <c r="C85" s="3"/>
@@ -2265,8 +2639,12 @@
       <c r="O85" s="3"/>
       <c r="P85" s="3"/>
       <c r="Q85" s="3"/>
-    </row>
-    <row r="86" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R85" s="3"/>
+      <c r="S85" s="3"/>
+      <c r="T85" s="3"/>
+      <c r="U85" s="3"/>
+    </row>
+    <row r="86" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A86" s="3"/>
       <c r="B86" s="3"/>
       <c r="C86" s="3"/>
@@ -2284,8 +2662,12 @@
       <c r="O86" s="3"/>
       <c r="P86" s="3"/>
       <c r="Q86" s="3"/>
-    </row>
-    <row r="87" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R86" s="3"/>
+      <c r="S86" s="3"/>
+      <c r="T86" s="3"/>
+      <c r="U86" s="3"/>
+    </row>
+    <row r="87" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A87" s="3"/>
       <c r="B87" s="3"/>
       <c r="C87" s="3"/>
@@ -2303,8 +2685,12 @@
       <c r="O87" s="3"/>
       <c r="P87" s="3"/>
       <c r="Q87" s="3"/>
-    </row>
-    <row r="88" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R87" s="3"/>
+      <c r="S87" s="3"/>
+      <c r="T87" s="3"/>
+      <c r="U87" s="3"/>
+    </row>
+    <row r="88" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A88" s="3"/>
       <c r="B88" s="3"/>
       <c r="C88" s="3"/>
@@ -2322,8 +2708,12 @@
       <c r="O88" s="3"/>
       <c r="P88" s="3"/>
       <c r="Q88" s="3"/>
-    </row>
-    <row r="89" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R88" s="3"/>
+      <c r="S88" s="3"/>
+      <c r="T88" s="3"/>
+      <c r="U88" s="3"/>
+    </row>
+    <row r="89" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A89" s="3"/>
       <c r="B89" s="3"/>
       <c r="C89" s="3"/>
@@ -2341,8 +2731,12 @@
       <c r="O89" s="3"/>
       <c r="P89" s="3"/>
       <c r="Q89" s="3"/>
-    </row>
-    <row r="90" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R89" s="3"/>
+      <c r="S89" s="3"/>
+      <c r="T89" s="3"/>
+      <c r="U89" s="3"/>
+    </row>
+    <row r="90" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A90" s="3"/>
       <c r="B90" s="3"/>
       <c r="C90" s="3"/>
@@ -2360,8 +2754,12 @@
       <c r="O90" s="3"/>
       <c r="P90" s="3"/>
       <c r="Q90" s="3"/>
-    </row>
-    <row r="91" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R90" s="3"/>
+      <c r="S90" s="3"/>
+      <c r="T90" s="3"/>
+      <c r="U90" s="3"/>
+    </row>
+    <row r="91" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A91" s="3"/>
       <c r="B91" s="3"/>
       <c r="C91" s="3"/>
@@ -2379,8 +2777,12 @@
       <c r="O91" s="3"/>
       <c r="P91" s="3"/>
       <c r="Q91" s="3"/>
-    </row>
-    <row r="92" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R91" s="3"/>
+      <c r="S91" s="3"/>
+      <c r="T91" s="3"/>
+      <c r="U91" s="3"/>
+    </row>
+    <row r="92" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A92" s="3"/>
       <c r="B92" s="3"/>
       <c r="C92" s="3"/>
@@ -2398,8 +2800,12 @@
       <c r="O92" s="3"/>
       <c r="P92" s="3"/>
       <c r="Q92" s="3"/>
-    </row>
-    <row r="93" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R92" s="3"/>
+      <c r="S92" s="3"/>
+      <c r="T92" s="3"/>
+      <c r="U92" s="3"/>
+    </row>
+    <row r="93" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A93" s="3"/>
       <c r="B93" s="3"/>
       <c r="C93" s="3"/>
@@ -2417,8 +2823,12 @@
       <c r="O93" s="3"/>
       <c r="P93" s="3"/>
       <c r="Q93" s="3"/>
-    </row>
-    <row r="94" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R93" s="3"/>
+      <c r="S93" s="3"/>
+      <c r="T93" s="3"/>
+      <c r="U93" s="3"/>
+    </row>
+    <row r="94" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A94" s="3"/>
       <c r="B94" s="3"/>
       <c r="C94" s="3"/>
@@ -2436,8 +2846,12 @@
       <c r="O94" s="3"/>
       <c r="P94" s="3"/>
       <c r="Q94" s="3"/>
-    </row>
-    <row r="95" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R94" s="3"/>
+      <c r="S94" s="3"/>
+      <c r="T94" s="3"/>
+      <c r="U94" s="3"/>
+    </row>
+    <row r="95" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A95" s="3"/>
       <c r="B95" s="3"/>
       <c r="C95" s="3"/>
@@ -2455,8 +2869,12 @@
       <c r="O95" s="3"/>
       <c r="P95" s="3"/>
       <c r="Q95" s="3"/>
-    </row>
-    <row r="96" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R95" s="3"/>
+      <c r="S95" s="3"/>
+      <c r="T95" s="3"/>
+      <c r="U95" s="3"/>
+    </row>
+    <row r="96" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A96" s="3"/>
       <c r="B96" s="3"/>
       <c r="C96" s="3"/>
@@ -2474,8 +2892,12 @@
       <c r="O96" s="3"/>
       <c r="P96" s="3"/>
       <c r="Q96" s="3"/>
-    </row>
-    <row r="97" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R96" s="3"/>
+      <c r="S96" s="3"/>
+      <c r="T96" s="3"/>
+      <c r="U96" s="3"/>
+    </row>
+    <row r="97" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A97" s="3"/>
       <c r="B97" s="3"/>
       <c r="C97" s="3"/>
@@ -2493,8 +2915,12 @@
       <c r="O97" s="3"/>
       <c r="P97" s="3"/>
       <c r="Q97" s="3"/>
-    </row>
-    <row r="98" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R97" s="3"/>
+      <c r="S97" s="3"/>
+      <c r="T97" s="3"/>
+      <c r="U97" s="3"/>
+    </row>
+    <row r="98" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
       <c r="B98" s="3"/>
       <c r="C98" s="3"/>
@@ -2512,8 +2938,12 @@
       <c r="O98" s="3"/>
       <c r="P98" s="3"/>
       <c r="Q98" s="3"/>
-    </row>
-    <row r="99" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R98" s="3"/>
+      <c r="S98" s="3"/>
+      <c r="T98" s="3"/>
+      <c r="U98" s="3"/>
+    </row>
+    <row r="99" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
       <c r="B99" s="3"/>
       <c r="C99" s="3"/>
@@ -2531,8 +2961,12 @@
       <c r="O99" s="3"/>
       <c r="P99" s="3"/>
       <c r="Q99" s="3"/>
-    </row>
-    <row r="100" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R99" s="3"/>
+      <c r="S99" s="3"/>
+      <c r="T99" s="3"/>
+      <c r="U99" s="3"/>
+    </row>
+    <row r="100" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
       <c r="B100" s="3"/>
       <c r="C100" s="3"/>
@@ -2550,8 +2984,12 @@
       <c r="O100" s="3"/>
       <c r="P100" s="3"/>
       <c r="Q100" s="3"/>
-    </row>
-    <row r="101" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R100" s="3"/>
+      <c r="S100" s="3"/>
+      <c r="T100" s="3"/>
+      <c r="U100" s="3"/>
+    </row>
+    <row r="101" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
       <c r="B101" s="3"/>
       <c r="C101" s="3"/>
@@ -2569,8 +3007,12 @@
       <c r="O101" s="3"/>
       <c r="P101" s="3"/>
       <c r="Q101" s="3"/>
-    </row>
-    <row r="102" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R101" s="3"/>
+      <c r="S101" s="3"/>
+      <c r="T101" s="3"/>
+      <c r="U101" s="3"/>
+    </row>
+    <row r="102" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A102" s="3"/>
       <c r="B102" s="3"/>
       <c r="C102" s="3"/>
@@ -2588,8 +3030,12 @@
       <c r="O102" s="3"/>
       <c r="P102" s="3"/>
       <c r="Q102" s="3"/>
-    </row>
-    <row r="103" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R102" s="3"/>
+      <c r="S102" s="3"/>
+      <c r="T102" s="3"/>
+      <c r="U102" s="3"/>
+    </row>
+    <row r="103" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
       <c r="B103" s="3"/>
       <c r="C103" s="3"/>
@@ -2607,8 +3053,12 @@
       <c r="O103" s="3"/>
       <c r="P103" s="3"/>
       <c r="Q103" s="3"/>
-    </row>
-    <row r="104" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R103" s="3"/>
+      <c r="S103" s="3"/>
+      <c r="T103" s="3"/>
+      <c r="U103" s="3"/>
+    </row>
+    <row r="104" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
       <c r="B104" s="3"/>
       <c r="C104" s="3"/>
@@ -2626,8 +3076,12 @@
       <c r="O104" s="3"/>
       <c r="P104" s="3"/>
       <c r="Q104" s="3"/>
-    </row>
-    <row r="105" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R104" s="3"/>
+      <c r="S104" s="3"/>
+      <c r="T104" s="3"/>
+      <c r="U104" s="3"/>
+    </row>
+    <row r="105" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
       <c r="B105" s="3"/>
       <c r="C105" s="3"/>
@@ -2645,8 +3099,12 @@
       <c r="O105" s="3"/>
       <c r="P105" s="3"/>
       <c r="Q105" s="3"/>
-    </row>
-    <row r="106" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R105" s="3"/>
+      <c r="S105" s="3"/>
+      <c r="T105" s="3"/>
+      <c r="U105" s="3"/>
+    </row>
+    <row r="106" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A106" s="3"/>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
@@ -2664,8 +3122,12 @@
       <c r="O106" s="3"/>
       <c r="P106" s="3"/>
       <c r="Q106" s="3"/>
-    </row>
-    <row r="107" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R106" s="3"/>
+      <c r="S106" s="3"/>
+      <c r="T106" s="3"/>
+      <c r="U106" s="3"/>
+    </row>
+    <row r="107" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
       <c r="B107" s="3"/>
       <c r="C107" s="3"/>
@@ -2683,8 +3145,12 @@
       <c r="O107" s="3"/>
       <c r="P107" s="3"/>
       <c r="Q107" s="3"/>
-    </row>
-    <row r="108" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R107" s="3"/>
+      <c r="S107" s="3"/>
+      <c r="T107" s="3"/>
+      <c r="U107" s="3"/>
+    </row>
+    <row r="108" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
       <c r="B108" s="3"/>
       <c r="C108" s="3"/>
@@ -2702,8 +3168,12 @@
       <c r="O108" s="3"/>
       <c r="P108" s="3"/>
       <c r="Q108" s="3"/>
-    </row>
-    <row r="109" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R108" s="3"/>
+      <c r="S108" s="3"/>
+      <c r="T108" s="3"/>
+      <c r="U108" s="3"/>
+    </row>
+    <row r="109" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
       <c r="B109" s="3"/>
       <c r="C109" s="3"/>
@@ -2721,8 +3191,12 @@
       <c r="O109" s="3"/>
       <c r="P109" s="3"/>
       <c r="Q109" s="3"/>
-    </row>
-    <row r="110" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R109" s="3"/>
+      <c r="S109" s="3"/>
+      <c r="T109" s="3"/>
+      <c r="U109" s="3"/>
+    </row>
+    <row r="110" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
       <c r="B110" s="3"/>
       <c r="C110" s="3"/>
@@ -2740,8 +3214,12 @@
       <c r="O110" s="3"/>
       <c r="P110" s="3"/>
       <c r="Q110" s="3"/>
-    </row>
-    <row r="111" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R110" s="3"/>
+      <c r="S110" s="3"/>
+      <c r="T110" s="3"/>
+      <c r="U110" s="3"/>
+    </row>
+    <row r="111" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
       <c r="B111" s="3"/>
       <c r="C111" s="3"/>
@@ -2759,8 +3237,12 @@
       <c r="O111" s="3"/>
       <c r="P111" s="3"/>
       <c r="Q111" s="3"/>
-    </row>
-    <row r="112" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R111" s="3"/>
+      <c r="S111" s="3"/>
+      <c r="T111" s="3"/>
+      <c r="U111" s="3"/>
+    </row>
+    <row r="112" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
       <c r="B112" s="3"/>
       <c r="C112" s="3"/>
@@ -2778,8 +3260,12 @@
       <c r="O112" s="3"/>
       <c r="P112" s="3"/>
       <c r="Q112" s="3"/>
-    </row>
-    <row r="113" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R112" s="3"/>
+      <c r="S112" s="3"/>
+      <c r="T112" s="3"/>
+      <c r="U112" s="3"/>
+    </row>
+    <row r="113" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A113" s="3"/>
       <c r="B113" s="3"/>
       <c r="C113" s="3"/>
@@ -2797,8 +3283,12 @@
       <c r="O113" s="3"/>
       <c r="P113" s="3"/>
       <c r="Q113" s="3"/>
-    </row>
-    <row r="114" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R113" s="3"/>
+      <c r="S113" s="3"/>
+      <c r="T113" s="3"/>
+      <c r="U113" s="3"/>
+    </row>
+    <row r="114" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A114" s="3"/>
       <c r="B114" s="3"/>
       <c r="C114" s="3"/>
@@ -2816,8 +3306,12 @@
       <c r="O114" s="3"/>
       <c r="P114" s="3"/>
       <c r="Q114" s="3"/>
-    </row>
-    <row r="115" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R114" s="3"/>
+      <c r="S114" s="3"/>
+      <c r="T114" s="3"/>
+      <c r="U114" s="3"/>
+    </row>
+    <row r="115" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A115" s="3"/>
       <c r="B115" s="3"/>
       <c r="C115" s="3"/>
@@ -2835,8 +3329,12 @@
       <c r="O115" s="3"/>
       <c r="P115" s="3"/>
       <c r="Q115" s="3"/>
-    </row>
-    <row r="116" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R115" s="3"/>
+      <c r="S115" s="3"/>
+      <c r="T115" s="3"/>
+      <c r="U115" s="3"/>
+    </row>
+    <row r="116" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A116" s="3"/>
       <c r="B116" s="3"/>
       <c r="C116" s="3"/>
@@ -2854,8 +3352,12 @@
       <c r="O116" s="3"/>
       <c r="P116" s="3"/>
       <c r="Q116" s="3"/>
-    </row>
-    <row r="117" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R116" s="3"/>
+      <c r="S116" s="3"/>
+      <c r="T116" s="3"/>
+      <c r="U116" s="3"/>
+    </row>
+    <row r="117" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A117" s="3"/>
       <c r="B117" s="3"/>
       <c r="C117" s="3"/>
@@ -2873,8 +3375,12 @@
       <c r="O117" s="3"/>
       <c r="P117" s="3"/>
       <c r="Q117" s="3"/>
-    </row>
-    <row r="118" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R117" s="3"/>
+      <c r="S117" s="3"/>
+      <c r="T117" s="3"/>
+      <c r="U117" s="3"/>
+    </row>
+    <row r="118" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A118" s="3"/>
       <c r="B118" s="3"/>
       <c r="C118" s="3"/>
@@ -2892,8 +3398,12 @@
       <c r="O118" s="3"/>
       <c r="P118" s="3"/>
       <c r="Q118" s="3"/>
-    </row>
-    <row r="119" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R118" s="3"/>
+      <c r="S118" s="3"/>
+      <c r="T118" s="3"/>
+      <c r="U118" s="3"/>
+    </row>
+    <row r="119" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A119" s="3"/>
       <c r="B119" s="3"/>
       <c r="C119" s="3"/>
@@ -2911,8 +3421,12 @@
       <c r="O119" s="3"/>
       <c r="P119" s="3"/>
       <c r="Q119" s="3"/>
-    </row>
-    <row r="120" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R119" s="3"/>
+      <c r="S119" s="3"/>
+      <c r="T119" s="3"/>
+      <c r="U119" s="3"/>
+    </row>
+    <row r="120" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A120" s="3"/>
       <c r="B120" s="3"/>
       <c r="C120" s="3"/>
@@ -2930,8 +3444,12 @@
       <c r="O120" s="3"/>
       <c r="P120" s="3"/>
       <c r="Q120" s="3"/>
-    </row>
-    <row r="121" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R120" s="3"/>
+      <c r="S120" s="3"/>
+      <c r="T120" s="3"/>
+      <c r="U120" s="3"/>
+    </row>
+    <row r="121" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A121" s="3"/>
       <c r="B121" s="3"/>
       <c r="C121" s="3"/>
@@ -2949,8 +3467,12 @@
       <c r="O121" s="3"/>
       <c r="P121" s="3"/>
       <c r="Q121" s="3"/>
-    </row>
-    <row r="122" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R121" s="3"/>
+      <c r="S121" s="3"/>
+      <c r="T121" s="3"/>
+      <c r="U121" s="3"/>
+    </row>
+    <row r="122" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A122" s="3"/>
       <c r="B122" s="3"/>
       <c r="C122" s="3"/>
@@ -2968,8 +3490,12 @@
       <c r="O122" s="3"/>
       <c r="P122" s="3"/>
       <c r="Q122" s="3"/>
-    </row>
-    <row r="123" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R122" s="3"/>
+      <c r="S122" s="3"/>
+      <c r="T122" s="3"/>
+      <c r="U122" s="3"/>
+    </row>
+    <row r="123" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A123" s="3"/>
       <c r="B123" s="3"/>
       <c r="C123" s="3"/>
@@ -2987,8 +3513,12 @@
       <c r="O123" s="3"/>
       <c r="P123" s="3"/>
       <c r="Q123" s="3"/>
-    </row>
-    <row r="124" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R123" s="3"/>
+      <c r="S123" s="3"/>
+      <c r="T123" s="3"/>
+      <c r="U123" s="3"/>
+    </row>
+    <row r="124" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A124" s="3"/>
       <c r="B124" s="3"/>
       <c r="C124" s="3"/>
@@ -3006,8 +3536,12 @@
       <c r="O124" s="3"/>
       <c r="P124" s="3"/>
       <c r="Q124" s="3"/>
-    </row>
-    <row r="125" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R124" s="3"/>
+      <c r="S124" s="3"/>
+      <c r="T124" s="3"/>
+      <c r="U124" s="3"/>
+    </row>
+    <row r="125" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A125" s="3"/>
       <c r="B125" s="3"/>
       <c r="C125" s="3"/>
@@ -3025,8 +3559,12 @@
       <c r="O125" s="3"/>
       <c r="P125" s="3"/>
       <c r="Q125" s="3"/>
-    </row>
-    <row r="126" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R125" s="3"/>
+      <c r="S125" s="3"/>
+      <c r="T125" s="3"/>
+      <c r="U125" s="3"/>
+    </row>
+    <row r="126" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A126" s="3"/>
       <c r="B126" s="3"/>
       <c r="C126" s="3"/>
@@ -3044,8 +3582,12 @@
       <c r="O126" s="3"/>
       <c r="P126" s="3"/>
       <c r="Q126" s="3"/>
-    </row>
-    <row r="127" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R126" s="3"/>
+      <c r="S126" s="3"/>
+      <c r="T126" s="3"/>
+      <c r="U126" s="3"/>
+    </row>
+    <row r="127" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A127" s="3"/>
       <c r="B127" s="3"/>
       <c r="C127" s="3"/>
@@ -3063,8 +3605,12 @@
       <c r="O127" s="3"/>
       <c r="P127" s="3"/>
       <c r="Q127" s="3"/>
-    </row>
-    <row r="128" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R127" s="3"/>
+      <c r="S127" s="3"/>
+      <c r="T127" s="3"/>
+      <c r="U127" s="3"/>
+    </row>
+    <row r="128" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A128" s="3"/>
       <c r="B128" s="3"/>
       <c r="C128" s="3"/>
@@ -3082,8 +3628,12 @@
       <c r="O128" s="3"/>
       <c r="P128" s="3"/>
       <c r="Q128" s="3"/>
-    </row>
-    <row r="129" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R128" s="3"/>
+      <c r="S128" s="3"/>
+      <c r="T128" s="3"/>
+      <c r="U128" s="3"/>
+    </row>
+    <row r="129" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A129" s="3"/>
       <c r="B129" s="3"/>
       <c r="C129" s="3"/>
@@ -3101,8 +3651,12 @@
       <c r="O129" s="3"/>
       <c r="P129" s="3"/>
       <c r="Q129" s="3"/>
-    </row>
-    <row r="130" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R129" s="3"/>
+      <c r="S129" s="3"/>
+      <c r="T129" s="3"/>
+      <c r="U129" s="3"/>
+    </row>
+    <row r="130" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A130" s="3"/>
       <c r="B130" s="3"/>
       <c r="C130" s="3"/>
@@ -3120,8 +3674,12 @@
       <c r="O130" s="3"/>
       <c r="P130" s="3"/>
       <c r="Q130" s="3"/>
-    </row>
-    <row r="131" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R130" s="3"/>
+      <c r="S130" s="3"/>
+      <c r="T130" s="3"/>
+      <c r="U130" s="3"/>
+    </row>
+    <row r="131" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="3"/>
       <c r="B131" s="3"/>
       <c r="C131" s="3"/>
@@ -3139,8 +3697,12 @@
       <c r="O131" s="3"/>
       <c r="P131" s="3"/>
       <c r="Q131" s="3"/>
-    </row>
-    <row r="132" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R131" s="3"/>
+      <c r="S131" s="3"/>
+      <c r="T131" s="3"/>
+      <c r="U131" s="3"/>
+    </row>
+    <row r="132" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="3"/>
       <c r="B132" s="3"/>
       <c r="C132" s="3"/>
@@ -3158,8 +3720,12 @@
       <c r="O132" s="3"/>
       <c r="P132" s="3"/>
       <c r="Q132" s="3"/>
-    </row>
-    <row r="133" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R132" s="3"/>
+      <c r="S132" s="3"/>
+      <c r="T132" s="3"/>
+      <c r="U132" s="3"/>
+    </row>
+    <row r="133" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="3"/>
       <c r="B133" s="3"/>
       <c r="C133" s="3"/>
@@ -3177,8 +3743,12 @@
       <c r="O133" s="3"/>
       <c r="P133" s="3"/>
       <c r="Q133" s="3"/>
-    </row>
-    <row r="134" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R133" s="3"/>
+      <c r="S133" s="3"/>
+      <c r="T133" s="3"/>
+      <c r="U133" s="3"/>
+    </row>
+    <row r="134" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="3"/>
       <c r="B134" s="3"/>
       <c r="C134" s="3"/>
@@ -3196,8 +3766,12 @@
       <c r="O134" s="3"/>
       <c r="P134" s="3"/>
       <c r="Q134" s="3"/>
-    </row>
-    <row r="135" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R134" s="3"/>
+      <c r="S134" s="3"/>
+      <c r="T134" s="3"/>
+      <c r="U134" s="3"/>
+    </row>
+    <row r="135" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="3"/>
       <c r="B135" s="3"/>
       <c r="C135" s="3"/>
@@ -3215,8 +3789,12 @@
       <c r="O135" s="3"/>
       <c r="P135" s="3"/>
       <c r="Q135" s="3"/>
-    </row>
-    <row r="136" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R135" s="3"/>
+      <c r="S135" s="3"/>
+      <c r="T135" s="3"/>
+      <c r="U135" s="3"/>
+    </row>
+    <row r="136" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="3"/>
       <c r="B136" s="3"/>
       <c r="C136" s="3"/>
@@ -3234,8 +3812,12 @@
       <c r="O136" s="3"/>
       <c r="P136" s="3"/>
       <c r="Q136" s="3"/>
-    </row>
-    <row r="137" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R136" s="3"/>
+      <c r="S136" s="3"/>
+      <c r="T136" s="3"/>
+      <c r="U136" s="3"/>
+    </row>
+    <row r="137" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A137" s="3"/>
       <c r="B137" s="3"/>
       <c r="C137" s="3"/>
@@ -3253,8 +3835,12 @@
       <c r="O137" s="3"/>
       <c r="P137" s="3"/>
       <c r="Q137" s="3"/>
-    </row>
-    <row r="138" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R137" s="3"/>
+      <c r="S137" s="3"/>
+      <c r="T137" s="3"/>
+      <c r="U137" s="3"/>
+    </row>
+    <row r="138" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A138" s="3"/>
       <c r="B138" s="3"/>
       <c r="C138" s="3"/>
@@ -3272,8 +3858,12 @@
       <c r="O138" s="3"/>
       <c r="P138" s="3"/>
       <c r="Q138" s="3"/>
-    </row>
-    <row r="139" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R138" s="3"/>
+      <c r="S138" s="3"/>
+      <c r="T138" s="3"/>
+      <c r="U138" s="3"/>
+    </row>
+    <row r="139" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A139" s="3"/>
       <c r="B139" s="3"/>
       <c r="C139" s="3"/>
@@ -3291,8 +3881,12 @@
       <c r="O139" s="3"/>
       <c r="P139" s="3"/>
       <c r="Q139" s="3"/>
-    </row>
-    <row r="140" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R139" s="3"/>
+      <c r="S139" s="3"/>
+      <c r="T139" s="3"/>
+      <c r="U139" s="3"/>
+    </row>
+    <row r="140" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A140" s="3"/>
       <c r="B140" s="3"/>
       <c r="C140" s="3"/>
@@ -3310,8 +3904,12 @@
       <c r="O140" s="3"/>
       <c r="P140" s="3"/>
       <c r="Q140" s="3"/>
-    </row>
-    <row r="141" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R140" s="3"/>
+      <c r="S140" s="3"/>
+      <c r="T140" s="3"/>
+      <c r="U140" s="3"/>
+    </row>
+    <row r="141" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A141" s="3"/>
       <c r="B141" s="3"/>
       <c r="C141" s="3"/>
@@ -3329,8 +3927,12 @@
       <c r="O141" s="3"/>
       <c r="P141" s="3"/>
       <c r="Q141" s="3"/>
-    </row>
-    <row r="142" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R141" s="3"/>
+      <c r="S141" s="3"/>
+      <c r="T141" s="3"/>
+      <c r="U141" s="3"/>
+    </row>
+    <row r="142" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A142" s="3"/>
       <c r="B142" s="3"/>
       <c r="C142" s="3"/>
@@ -3348,8 +3950,12 @@
       <c r="O142" s="3"/>
       <c r="P142" s="3"/>
       <c r="Q142" s="3"/>
-    </row>
-    <row r="143" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R142" s="3"/>
+      <c r="S142" s="3"/>
+      <c r="T142" s="3"/>
+      <c r="U142" s="3"/>
+    </row>
+    <row r="143" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A143" s="3"/>
       <c r="B143" s="3"/>
       <c r="C143" s="3"/>
@@ -3367,8 +3973,12 @@
       <c r="O143" s="3"/>
       <c r="P143" s="3"/>
       <c r="Q143" s="3"/>
-    </row>
-    <row r="144" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R143" s="3"/>
+      <c r="S143" s="3"/>
+      <c r="T143" s="3"/>
+      <c r="U143" s="3"/>
+    </row>
+    <row r="144" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A144" s="3"/>
       <c r="B144" s="3"/>
       <c r="C144" s="3"/>
@@ -3386,8 +3996,12 @@
       <c r="O144" s="3"/>
       <c r="P144" s="3"/>
       <c r="Q144" s="3"/>
-    </row>
-    <row r="145" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R144" s="3"/>
+      <c r="S144" s="3"/>
+      <c r="T144" s="3"/>
+      <c r="U144" s="3"/>
+    </row>
+    <row r="145" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A145" s="3"/>
       <c r="B145" s="3"/>
       <c r="C145" s="3"/>
@@ -3405,8 +4019,12 @@
       <c r="O145" s="3"/>
       <c r="P145" s="3"/>
       <c r="Q145" s="3"/>
-    </row>
-    <row r="146" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R145" s="3"/>
+      <c r="S145" s="3"/>
+      <c r="T145" s="3"/>
+      <c r="U145" s="3"/>
+    </row>
+    <row r="146" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A146" s="3"/>
       <c r="B146" s="3"/>
       <c r="C146" s="3"/>
@@ -3424,8 +4042,12 @@
       <c r="O146" s="3"/>
       <c r="P146" s="3"/>
       <c r="Q146" s="3"/>
-    </row>
-    <row r="147" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R146" s="3"/>
+      <c r="S146" s="3"/>
+      <c r="T146" s="3"/>
+      <c r="U146" s="3"/>
+    </row>
+    <row r="147" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A147" s="3"/>
       <c r="B147" s="3"/>
       <c r="C147" s="3"/>
@@ -3443,8 +4065,12 @@
       <c r="O147" s="3"/>
       <c r="P147" s="3"/>
       <c r="Q147" s="3"/>
-    </row>
-    <row r="148" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R147" s="3"/>
+      <c r="S147" s="3"/>
+      <c r="T147" s="3"/>
+      <c r="U147" s="3"/>
+    </row>
+    <row r="148" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A148" s="3"/>
       <c r="B148" s="3"/>
       <c r="C148" s="3"/>
@@ -3462,8 +4088,12 @@
       <c r="O148" s="3"/>
       <c r="P148" s="3"/>
       <c r="Q148" s="3"/>
-    </row>
-    <row r="149" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R148" s="3"/>
+      <c r="S148" s="3"/>
+      <c r="T148" s="3"/>
+      <c r="U148" s="3"/>
+    </row>
+    <row r="149" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A149" s="3"/>
       <c r="B149" s="3"/>
       <c r="C149" s="3"/>
@@ -3481,8 +4111,12 @@
       <c r="O149" s="3"/>
       <c r="P149" s="3"/>
       <c r="Q149" s="3"/>
-    </row>
-    <row r="150" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R149" s="3"/>
+      <c r="S149" s="3"/>
+      <c r="T149" s="3"/>
+      <c r="U149" s="3"/>
+    </row>
+    <row r="150" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A150" s="3"/>
       <c r="B150" s="3"/>
       <c r="C150" s="3"/>
@@ -3500,8 +4134,12 @@
       <c r="O150" s="3"/>
       <c r="P150" s="3"/>
       <c r="Q150" s="3"/>
-    </row>
-    <row r="151" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R150" s="3"/>
+      <c r="S150" s="3"/>
+      <c r="T150" s="3"/>
+      <c r="U150" s="3"/>
+    </row>
+    <row r="151" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A151" s="3"/>
       <c r="B151" s="3"/>
       <c r="C151" s="3"/>
@@ -3519,8 +4157,12 @@
       <c r="O151" s="3"/>
       <c r="P151" s="3"/>
       <c r="Q151" s="3"/>
-    </row>
-    <row r="152" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R151" s="3"/>
+      <c r="S151" s="3"/>
+      <c r="T151" s="3"/>
+      <c r="U151" s="3"/>
+    </row>
+    <row r="152" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A152" s="3"/>
       <c r="B152" s="3"/>
       <c r="C152" s="3"/>
@@ -3538,8 +4180,12 @@
       <c r="O152" s="3"/>
       <c r="P152" s="3"/>
       <c r="Q152" s="3"/>
-    </row>
-    <row r="153" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R152" s="3"/>
+      <c r="S152" s="3"/>
+      <c r="T152" s="3"/>
+      <c r="U152" s="3"/>
+    </row>
+    <row r="153" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A153" s="3"/>
       <c r="B153" s="3"/>
       <c r="C153" s="3"/>
@@ -3557,8 +4203,12 @@
       <c r="O153" s="3"/>
       <c r="P153" s="3"/>
       <c r="Q153" s="3"/>
-    </row>
-    <row r="154" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R153" s="3"/>
+      <c r="S153" s="3"/>
+      <c r="T153" s="3"/>
+      <c r="U153" s="3"/>
+    </row>
+    <row r="154" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A154" s="3"/>
       <c r="B154" s="3"/>
       <c r="C154" s="3"/>
@@ -3576,8 +4226,12 @@
       <c r="O154" s="3"/>
       <c r="P154" s="3"/>
       <c r="Q154" s="3"/>
-    </row>
-    <row r="155" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R154" s="3"/>
+      <c r="S154" s="3"/>
+      <c r="T154" s="3"/>
+      <c r="U154" s="3"/>
+    </row>
+    <row r="155" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A155" s="3"/>
       <c r="B155" s="3"/>
       <c r="C155" s="3"/>
@@ -3595,8 +4249,12 @@
       <c r="O155" s="3"/>
       <c r="P155" s="3"/>
       <c r="Q155" s="3"/>
-    </row>
-    <row r="156" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R155" s="3"/>
+      <c r="S155" s="3"/>
+      <c r="T155" s="3"/>
+      <c r="U155" s="3"/>
+    </row>
+    <row r="156" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A156" s="3"/>
       <c r="B156" s="3"/>
       <c r="C156" s="3"/>
@@ -3614,8 +4272,12 @@
       <c r="O156" s="3"/>
       <c r="P156" s="3"/>
       <c r="Q156" s="3"/>
-    </row>
-    <row r="157" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R156" s="3"/>
+      <c r="S156" s="3"/>
+      <c r="T156" s="3"/>
+      <c r="U156" s="3"/>
+    </row>
+    <row r="157" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A157" s="3"/>
       <c r="B157" s="3"/>
       <c r="C157" s="3"/>
@@ -3633,8 +4295,12 @@
       <c r="O157" s="3"/>
       <c r="P157" s="3"/>
       <c r="Q157" s="3"/>
-    </row>
-    <row r="158" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R157" s="3"/>
+      <c r="S157" s="3"/>
+      <c r="T157" s="3"/>
+      <c r="U157" s="3"/>
+    </row>
+    <row r="158" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A158" s="3"/>
       <c r="B158" s="3"/>
       <c r="C158" s="3"/>
@@ -3652,8 +4318,12 @@
       <c r="O158" s="3"/>
       <c r="P158" s="3"/>
       <c r="Q158" s="3"/>
-    </row>
-    <row r="159" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R158" s="3"/>
+      <c r="S158" s="3"/>
+      <c r="T158" s="3"/>
+      <c r="U158" s="3"/>
+    </row>
+    <row r="159" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A159" s="3"/>
       <c r="B159" s="3"/>
       <c r="C159" s="3"/>
@@ -3671,8 +4341,12 @@
       <c r="O159" s="3"/>
       <c r="P159" s="3"/>
       <c r="Q159" s="3"/>
-    </row>
-    <row r="160" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R159" s="3"/>
+      <c r="S159" s="3"/>
+      <c r="T159" s="3"/>
+      <c r="U159" s="3"/>
+    </row>
+    <row r="160" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
       <c r="C160" s="3"/>
@@ -3690,8 +4364,12 @@
       <c r="O160" s="3"/>
       <c r="P160" s="3"/>
       <c r="Q160" s="3"/>
-    </row>
-    <row r="161" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R160" s="3"/>
+      <c r="S160" s="3"/>
+      <c r="T160" s="3"/>
+      <c r="U160" s="3"/>
+    </row>
+    <row r="161" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A161" s="3"/>
       <c r="B161" s="3"/>
       <c r="C161" s="3"/>
@@ -3709,8 +4387,12 @@
       <c r="O161" s="3"/>
       <c r="P161" s="3"/>
       <c r="Q161" s="3"/>
-    </row>
-    <row r="162" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R161" s="3"/>
+      <c r="S161" s="3"/>
+      <c r="T161" s="3"/>
+      <c r="U161" s="3"/>
+    </row>
+    <row r="162" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
       <c r="C162" s="3"/>
@@ -3728,8 +4410,12 @@
       <c r="O162" s="3"/>
       <c r="P162" s="3"/>
       <c r="Q162" s="3"/>
-    </row>
-    <row r="163" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R162" s="3"/>
+      <c r="S162" s="3"/>
+      <c r="T162" s="3"/>
+      <c r="U162" s="3"/>
+    </row>
+    <row r="163" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
       <c r="C163" s="3"/>
@@ -3747,8 +4433,12 @@
       <c r="O163" s="3"/>
       <c r="P163" s="3"/>
       <c r="Q163" s="3"/>
-    </row>
-    <row r="164" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R163" s="3"/>
+      <c r="S163" s="3"/>
+      <c r="T163" s="3"/>
+      <c r="U163" s="3"/>
+    </row>
+    <row r="164" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A164" s="3"/>
       <c r="B164" s="3"/>
       <c r="C164" s="3"/>
@@ -3766,8 +4456,12 @@
       <c r="O164" s="3"/>
       <c r="P164" s="3"/>
       <c r="Q164" s="3"/>
-    </row>
-    <row r="165" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R164" s="3"/>
+      <c r="S164" s="3"/>
+      <c r="T164" s="3"/>
+      <c r="U164" s="3"/>
+    </row>
+    <row r="165" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
       <c r="C165" s="3"/>
@@ -3785,8 +4479,12 @@
       <c r="O165" s="3"/>
       <c r="P165" s="3"/>
       <c r="Q165" s="3"/>
-    </row>
-    <row r="166" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R165" s="3"/>
+      <c r="S165" s="3"/>
+      <c r="T165" s="3"/>
+      <c r="U165" s="3"/>
+    </row>
+    <row r="166" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
       <c r="C166" s="3"/>
@@ -3804,8 +4502,12 @@
       <c r="O166" s="3"/>
       <c r="P166" s="3"/>
       <c r="Q166" s="3"/>
-    </row>
-    <row r="167" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R166" s="3"/>
+      <c r="S166" s="3"/>
+      <c r="T166" s="3"/>
+      <c r="U166" s="3"/>
+    </row>
+    <row r="167" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
       <c r="C167" s="3"/>
@@ -3823,8 +4525,12 @@
       <c r="O167" s="3"/>
       <c r="P167" s="3"/>
       <c r="Q167" s="3"/>
-    </row>
-    <row r="168" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R167" s="3"/>
+      <c r="S167" s="3"/>
+      <c r="T167" s="3"/>
+      <c r="U167" s="3"/>
+    </row>
+    <row r="168" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="3"/>
@@ -3842,8 +4548,12 @@
       <c r="O168" s="3"/>
       <c r="P168" s="3"/>
       <c r="Q168" s="3"/>
-    </row>
-    <row r="169" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R168" s="3"/>
+      <c r="S168" s="3"/>
+      <c r="T168" s="3"/>
+      <c r="U168" s="3"/>
+    </row>
+    <row r="169" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="3"/>
@@ -3861,8 +4571,12 @@
       <c r="O169" s="3"/>
       <c r="P169" s="3"/>
       <c r="Q169" s="3"/>
-    </row>
-    <row r="170" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R169" s="3"/>
+      <c r="S169" s="3"/>
+      <c r="T169" s="3"/>
+      <c r="U169" s="3"/>
+    </row>
+    <row r="170" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
       <c r="C170" s="3"/>
@@ -3880,8 +4594,12 @@
       <c r="O170" s="3"/>
       <c r="P170" s="3"/>
       <c r="Q170" s="3"/>
-    </row>
-    <row r="171" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R170" s="3"/>
+      <c r="S170" s="3"/>
+      <c r="T170" s="3"/>
+      <c r="U170" s="3"/>
+    </row>
+    <row r="171" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="3"/>
@@ -3899,8 +4617,12 @@
       <c r="O171" s="3"/>
       <c r="P171" s="3"/>
       <c r="Q171" s="3"/>
-    </row>
-    <row r="172" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R171" s="3"/>
+      <c r="S171" s="3"/>
+      <c r="T171" s="3"/>
+      <c r="U171" s="3"/>
+    </row>
+    <row r="172" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="3"/>
@@ -3918,8 +4640,12 @@
       <c r="O172" s="3"/>
       <c r="P172" s="3"/>
       <c r="Q172" s="3"/>
-    </row>
-    <row r="173" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R172" s="3"/>
+      <c r="S172" s="3"/>
+      <c r="T172" s="3"/>
+      <c r="U172" s="3"/>
+    </row>
+    <row r="173" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="3"/>
@@ -3937,8 +4663,12 @@
       <c r="O173" s="3"/>
       <c r="P173" s="3"/>
       <c r="Q173" s="3"/>
-    </row>
-    <row r="174" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R173" s="3"/>
+      <c r="S173" s="3"/>
+      <c r="T173" s="3"/>
+      <c r="U173" s="3"/>
+    </row>
+    <row r="174" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="3"/>
@@ -3956,8 +4686,12 @@
       <c r="O174" s="3"/>
       <c r="P174" s="3"/>
       <c r="Q174" s="3"/>
-    </row>
-    <row r="175" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R174" s="3"/>
+      <c r="S174" s="3"/>
+      <c r="T174" s="3"/>
+      <c r="U174" s="3"/>
+    </row>
+    <row r="175" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="3"/>
@@ -3975,8 +4709,12 @@
       <c r="O175" s="3"/>
       <c r="P175" s="3"/>
       <c r="Q175" s="3"/>
-    </row>
-    <row r="176" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R175" s="3"/>
+      <c r="S175" s="3"/>
+      <c r="T175" s="3"/>
+      <c r="U175" s="3"/>
+    </row>
+    <row r="176" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="3"/>
@@ -3994,8 +4732,12 @@
       <c r="O176" s="3"/>
       <c r="P176" s="3"/>
       <c r="Q176" s="3"/>
-    </row>
-    <row r="177" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R176" s="3"/>
+      <c r="S176" s="3"/>
+      <c r="T176" s="3"/>
+      <c r="U176" s="3"/>
+    </row>
+    <row r="177" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="3"/>
@@ -4013,8 +4755,12 @@
       <c r="O177" s="3"/>
       <c r="P177" s="3"/>
       <c r="Q177" s="3"/>
-    </row>
-    <row r="178" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R177" s="3"/>
+      <c r="S177" s="3"/>
+      <c r="T177" s="3"/>
+      <c r="U177" s="3"/>
+    </row>
+    <row r="178" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="3"/>
@@ -4032,8 +4778,12 @@
       <c r="O178" s="3"/>
       <c r="P178" s="3"/>
       <c r="Q178" s="3"/>
-    </row>
-    <row r="179" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R178" s="3"/>
+      <c r="S178" s="3"/>
+      <c r="T178" s="3"/>
+      <c r="U178" s="3"/>
+    </row>
+    <row r="179" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="3"/>
@@ -4051,8 +4801,12 @@
       <c r="O179" s="3"/>
       <c r="P179" s="3"/>
       <c r="Q179" s="3"/>
-    </row>
-    <row r="180" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R179" s="3"/>
+      <c r="S179" s="3"/>
+      <c r="T179" s="3"/>
+      <c r="U179" s="3"/>
+    </row>
+    <row r="180" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
       <c r="C180" s="3"/>
@@ -4070,8 +4824,12 @@
       <c r="O180" s="3"/>
       <c r="P180" s="3"/>
       <c r="Q180" s="3"/>
-    </row>
-    <row r="181" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R180" s="3"/>
+      <c r="S180" s="3"/>
+      <c r="T180" s="3"/>
+      <c r="U180" s="3"/>
+    </row>
+    <row r="181" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
       <c r="C181" s="3"/>
@@ -4089,8 +4847,12 @@
       <c r="O181" s="3"/>
       <c r="P181" s="3"/>
       <c r="Q181" s="3"/>
-    </row>
-    <row r="182" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R181" s="3"/>
+      <c r="S181" s="3"/>
+      <c r="T181" s="3"/>
+      <c r="U181" s="3"/>
+    </row>
+    <row r="182" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
       <c r="C182" s="3"/>
@@ -4108,8 +4870,12 @@
       <c r="O182" s="3"/>
       <c r="P182" s="3"/>
       <c r="Q182" s="3"/>
-    </row>
-    <row r="183" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R182" s="3"/>
+      <c r="S182" s="3"/>
+      <c r="T182" s="3"/>
+      <c r="U182" s="3"/>
+    </row>
+    <row r="183" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
       <c r="C183" s="3"/>
@@ -4127,8 +4893,12 @@
       <c r="O183" s="3"/>
       <c r="P183" s="3"/>
       <c r="Q183" s="3"/>
-    </row>
-    <row r="184" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R183" s="3"/>
+      <c r="S183" s="3"/>
+      <c r="T183" s="3"/>
+      <c r="U183" s="3"/>
+    </row>
+    <row r="184" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="3"/>
@@ -4146,8 +4916,12 @@
       <c r="O184" s="3"/>
       <c r="P184" s="3"/>
       <c r="Q184" s="3"/>
-    </row>
-    <row r="185" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R184" s="3"/>
+      <c r="S184" s="3"/>
+      <c r="T184" s="3"/>
+      <c r="U184" s="3"/>
+    </row>
+    <row r="185" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="3"/>
@@ -4165,8 +4939,12 @@
       <c r="O185" s="3"/>
       <c r="P185" s="3"/>
       <c r="Q185" s="3"/>
-    </row>
-    <row r="186" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R185" s="3"/>
+      <c r="S185" s="3"/>
+      <c r="T185" s="3"/>
+      <c r="U185" s="3"/>
+    </row>
+    <row r="186" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="3"/>
@@ -4184,8 +4962,12 @@
       <c r="O186" s="3"/>
       <c r="P186" s="3"/>
       <c r="Q186" s="3"/>
-    </row>
-    <row r="187" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R186" s="3"/>
+      <c r="S186" s="3"/>
+      <c r="T186" s="3"/>
+      <c r="U186" s="3"/>
+    </row>
+    <row r="187" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="3"/>
@@ -4203,8 +4985,12 @@
       <c r="O187" s="3"/>
       <c r="P187" s="3"/>
       <c r="Q187" s="3"/>
-    </row>
-    <row r="188" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R187" s="3"/>
+      <c r="S187" s="3"/>
+      <c r="T187" s="3"/>
+      <c r="U187" s="3"/>
+    </row>
+    <row r="188" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="3"/>
@@ -4222,8 +5008,12 @@
       <c r="O188" s="3"/>
       <c r="P188" s="3"/>
       <c r="Q188" s="3"/>
-    </row>
-    <row r="189" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R188" s="3"/>
+      <c r="S188" s="3"/>
+      <c r="T188" s="3"/>
+      <c r="U188" s="3"/>
+    </row>
+    <row r="189" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="3"/>
@@ -4241,8 +5031,12 @@
       <c r="O189" s="3"/>
       <c r="P189" s="3"/>
       <c r="Q189" s="3"/>
-    </row>
-    <row r="190" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R189" s="3"/>
+      <c r="S189" s="3"/>
+      <c r="T189" s="3"/>
+      <c r="U189" s="3"/>
+    </row>
+    <row r="190" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="3"/>
@@ -4260,8 +5054,12 @@
       <c r="O190" s="3"/>
       <c r="P190" s="3"/>
       <c r="Q190" s="3"/>
-    </row>
-    <row r="191" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R190" s="3"/>
+      <c r="S190" s="3"/>
+      <c r="T190" s="3"/>
+      <c r="U190" s="3"/>
+    </row>
+    <row r="191" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="3"/>
@@ -4279,8 +5077,12 @@
       <c r="O191" s="3"/>
       <c r="P191" s="3"/>
       <c r="Q191" s="3"/>
-    </row>
-    <row r="192" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R191" s="3"/>
+      <c r="S191" s="3"/>
+      <c r="T191" s="3"/>
+      <c r="U191" s="3"/>
+    </row>
+    <row r="192" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="3"/>
@@ -4298,8 +5100,12 @@
       <c r="O192" s="3"/>
       <c r="P192" s="3"/>
       <c r="Q192" s="3"/>
-    </row>
-    <row r="193" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R192" s="3"/>
+      <c r="S192" s="3"/>
+      <c r="T192" s="3"/>
+      <c r="U192" s="3"/>
+    </row>
+    <row r="193" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A193" s="3"/>
       <c r="B193" s="3"/>
       <c r="C193" s="3"/>
@@ -4317,8 +5123,12 @@
       <c r="O193" s="3"/>
       <c r="P193" s="3"/>
       <c r="Q193" s="3"/>
-    </row>
-    <row r="194" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R193" s="3"/>
+      <c r="S193" s="3"/>
+      <c r="T193" s="3"/>
+      <c r="U193" s="3"/>
+    </row>
+    <row r="194" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A194" s="3"/>
       <c r="B194" s="3"/>
       <c r="C194" s="3"/>
@@ -4336,8 +5146,12 @@
       <c r="O194" s="3"/>
       <c r="P194" s="3"/>
       <c r="Q194" s="3"/>
-    </row>
-    <row r="195" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R194" s="3"/>
+      <c r="S194" s="3"/>
+      <c r="T194" s="3"/>
+      <c r="U194" s="3"/>
+    </row>
+    <row r="195" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A195" s="3"/>
       <c r="B195" s="3"/>
       <c r="C195" s="3"/>
@@ -4355,8 +5169,12 @@
       <c r="O195" s="3"/>
       <c r="P195" s="3"/>
       <c r="Q195" s="3"/>
-    </row>
-    <row r="196" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R195" s="3"/>
+      <c r="S195" s="3"/>
+      <c r="T195" s="3"/>
+      <c r="U195" s="3"/>
+    </row>
+    <row r="196" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A196" s="3"/>
       <c r="B196" s="3"/>
       <c r="C196" s="3"/>
@@ -4374,8 +5192,12 @@
       <c r="O196" s="3"/>
       <c r="P196" s="3"/>
       <c r="Q196" s="3"/>
-    </row>
-    <row r="197" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R196" s="3"/>
+      <c r="S196" s="3"/>
+      <c r="T196" s="3"/>
+      <c r="U196" s="3"/>
+    </row>
+    <row r="197" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A197" s="3"/>
       <c r="B197" s="3"/>
       <c r="C197" s="3"/>
@@ -4393,8 +5215,12 @@
       <c r="O197" s="3"/>
       <c r="P197" s="3"/>
       <c r="Q197" s="3"/>
-    </row>
-    <row r="198" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R197" s="3"/>
+      <c r="S197" s="3"/>
+      <c r="T197" s="3"/>
+      <c r="U197" s="3"/>
+    </row>
+    <row r="198" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A198" s="3"/>
       <c r="B198" s="3"/>
       <c r="C198" s="3"/>
@@ -4412,8 +5238,12 @@
       <c r="O198" s="3"/>
       <c r="P198" s="3"/>
       <c r="Q198" s="3"/>
-    </row>
-    <row r="199" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R198" s="3"/>
+      <c r="S198" s="3"/>
+      <c r="T198" s="3"/>
+      <c r="U198" s="3"/>
+    </row>
+    <row r="199" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A199" s="3"/>
       <c r="B199" s="3"/>
       <c r="C199" s="3"/>
@@ -4431,8 +5261,12 @@
       <c r="O199" s="3"/>
       <c r="P199" s="3"/>
       <c r="Q199" s="3"/>
-    </row>
-    <row r="200" ht="20" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="R199" s="3"/>
+      <c r="S199" s="3"/>
+      <c r="T199" s="3"/>
+      <c r="U199" s="3"/>
+    </row>
+    <row r="200" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A200" s="3"/>
       <c r="B200" s="3"/>
       <c r="C200" s="3"/>
@@ -4450,6 +5284,10 @@
       <c r="O200" s="3"/>
       <c r="P200" s="3"/>
       <c r="Q200" s="3"/>
+      <c r="R200" s="3"/>
+      <c r="S200" s="3"/>
+      <c r="T200" s="3"/>
+      <c r="U200" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix: add IT status example data to template row 3
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Import_Template.xlsx
+++ b/public/Import_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -125,6 +125,21 @@
   </si>
   <si>
     <t>pornpetch.n@redcross.or.th</t>
+  </si>
+  <si>
+    <t>ดำเนินการแล้ว</t>
+  </si>
+  <si>
+    <t>01/06/2568</t>
+  </si>
+  <si>
+    <t>ยังไม่ดำเนินการ</t>
+  </si>
+  <si>
+    <t>15/01/2569</t>
+  </si>
+  <si>
+    <t>ไม่พบบัญชี</t>
   </si>
 </sst>
 </file>
@@ -749,13 +764,25 @@
       <c r="M3" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="N3" s="3"/>
-      <c r="O3" s="3"/>
-      <c r="P3" s="3"/>
+      <c r="N3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="P3" s="3" t="s">
+        <v>40</v>
+      </c>
       <c r="Q3" s="3"/>
-      <c r="R3" s="3"/>
-      <c r="S3" s="3"/>
-      <c r="T3" s="3"/>
+      <c r="R3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="S3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="T3" s="3" t="s">
+        <v>42</v>
+      </c>
       <c r="U3" s="3"/>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
fix: store IT status as string instead of null, update template with dropdown and styling
- Migrate DB: null to ไม่พบบัญชี for fmis/eMeeting/software/phonebook
- Fix normalizeITStatus to return string (not null) for ไม่พบบัญชี
- Fix import CREATE/UPDATE paths to store ไม่พบบัญชี as string
- Fix filter and cleared logic to use string comparison instead of null check
- Fix frontend ITStatusCell, ITBadge, isFullyClosed to handle string value
- Fix IT_OPTS in Add/Edit forms to use ไม่พบบัญชี as actual value
- Update Import_Template.xlsx: TH Sarabun New font, dropdown validation, row 2 warning

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Import_Template.xlsx
+++ b/public/Import_Template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="44">
   <si>
     <t>ข้อมูลต้นทาง</t>
   </si>
@@ -88,6 +88,9 @@
     <t>วัน/เดือน/ปี พ.ศ.</t>
   </si>
   <si>
+    <t>⚠️ ลบแถวนี้ออกก่อนใช้งาน</t>
+  </si>
+  <si>
     <t>เจ้าหน้าที่, ชั่วคราว</t>
   </si>
   <si>
@@ -157,16 +160,19 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="14"/>
+      <name val="TH Sarabun New"/>
     </font>
     <font>
+      <b/>
       <i/>
-      <color rgb="FF6B7280"/>
-      <sz val="11"/>
-      <name val="TH SarabunPSK"/>
+      <color rgb="FFFF0000"/>
+      <sz val="14"/>
+      <name val="TH Sarabun New"/>
     </font>
     <font>
-      <sz val="12"/>
-      <name val="TH SarabunPSK"/>
+      <sz val="14"/>
+      <name val="TH Sarabun New"/>
     </font>
   </fonts>
   <fills count="5">
@@ -183,7 +189,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF9FAFB"/>
+        <fgColor rgb="FFFFD966"/>
       </patternFill>
     </fill>
     <fill>
@@ -685,11 +691,13 @@
         <v>24</v>
       </c>
       <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
@@ -697,31 +705,31 @@
         <v>24</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="P2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="P2" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="Q2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="R2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="R2" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="S2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="T2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>27</v>
-      </c>
       <c r="U2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:21" x14ac:dyDescent="0.25">
@@ -735,53 +743,53 @@
         <v>2599</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>29</v>
-      </c>
       <c r="M3" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N3" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="P3" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="Q3" s="3"/>
       <c r="R3" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="U3" s="3"/>
     </row>
@@ -5317,6 +5325,32 @@
       <c r="U200" s="3"/>
     </row>
   </sheetData>
+  <dataValidations count="8">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N10:N200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N3:N200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P10:P200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P3:P200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R10:R200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R3:R200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T10:T200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T3:T200">
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: add ไม่ทราบสถานะ as 4th IT status (treated as closed)
- employees.ts: refactor valid IT status list to VALID_IT_STATUSES constant,
  fix import UPDATE bug that was mapping ไม่พบบัญชี → null
- dashboard.ts: include ไม่ทราบสถานะ in cleared logic, add unknown counter
- reports.ts: include ไม่ทราบสถานะ in isItCleared, breakdown counter,
  Excel report adds column and purple styling
- AllRecordsPage: isFullyClosed, ITStatusCell, ITBadge, mobile badges,
  filter dropdown all updated with violet badge for ไม่ทราบสถานะ
- EditRecordModal, AddRecordPage: add to IT_OPTS dropdown
- ImportPage, UpdateITStatusPage: update hint text
- DashboardPage: add unknown counter with violet dot in breakdown bar
- Excel template: add ไม่ทราบสถานะ to dropdown validation

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Import_Template.xlsx
+++ b/public/Import_Template.xlsx
@@ -5327,28 +5327,28 @@
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N10:N200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="N3:N200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P10:P200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="P3:P200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R10:R200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="R3:R200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T10:T200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorStyle="warning" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือก: ดำเนินการแล้ว, ยังไม่ดำเนินการ หรือ ไม่พบบัญชี" sqref="T3:T200">
-      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี"</formula1>
+      <formula1>"ดำเนินการแล้ว,ยังไม่ดำเนินการ,ไม่พบบัญชี,ไม่ทราบสถานะ"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>